<commit_message>
Carga masiva de base de datos por FERNANDO (193 registros, 15/09/2026 13:33)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -3071,7 +3071,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>VICTORIA</t>
+          <t>MARIA VICTORIA</t>
         </is>
       </c>
       <c r="H11" s="1" t="n">
@@ -5687,7 +5687,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>VICTORIA</t>
+          <t>MARIA VICTORIA</t>
         </is>
       </c>
       <c r="H24" s="1" t="n">
@@ -20189,7 +20189,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>VICTORIA</t>
+          <t>MARIA VICTORIA</t>
         </is>
       </c>
       <c r="H83" s="1" t="n">
@@ -22763,7 +22763,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>VICTORIA</t>
+          <t>MARIA VICTORIA</t>
         </is>
       </c>
       <c r="H95" s="1" t="n">
@@ -39539,7 +39539,7 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>VICTORIA</t>
+          <t>MARIA VICTORIA</t>
         </is>
       </c>
       <c r="H184" s="1" t="n">

</xml_diff>

<commit_message>
Kanban: folio DC-AB009 → 📝 Reporte recibido
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -4769,12 +4769,12 @@
       <c r="U58" t="inlineStr"/>
       <c r="V58" t="inlineStr">
         <is>
-          <t>21/09/2026 14:15</t>
+          <t>21/09/2026 14:16</t>
         </is>
       </c>
       <c r="W58" t="inlineStr">
         <is>
-          <t>📤 Reportado al proveedor</t>
+          <t>📝 Reporte recibido</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Carga masiva (249+76+91 registros) 21/09/2026 14:55
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dsanver-my.sharepoint.com/personal/compras_dsanver_onmicrosoft_com/Documents/Documentos/FERNANDO TREVIÑO/Devoluciones/NV_001/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B2EDD2CD-A11A-4C02-9527-D1EA1C70CBE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="8_{B2EDD2CD-A11A-4C02-9527-D1EA1C70CBE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B1BD2E7-0DAD-432B-A15D-2DD2963CEA1A}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="datos- FOLIO DE GARANTIA" sheetId="1" r:id="rId1"/>
@@ -20,12 +20,25 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'NC PENDIENTES'!$B$1:$Y$92</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3317" uniqueCount="761">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3526" uniqueCount="761">
   <si>
     <t>MES DE DEVOLUCION</t>
   </si>
@@ -2315,7 +2328,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -2346,10 +2359,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2790,6 +2804,9 @@
       <c r="R2" t="s">
         <v>31</v>
       </c>
+      <c r="U2" s="3">
+        <v>46251</v>
+      </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
@@ -2840,6 +2857,9 @@
       <c r="R3" t="s">
         <v>38</v>
       </c>
+      <c r="U3" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W3" t="s">
         <v>39</v>
       </c>
@@ -2890,6 +2910,9 @@
       <c r="R4" t="s">
         <v>31</v>
       </c>
+      <c r="U4" s="3">
+        <v>46199</v>
+      </c>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
@@ -2940,6 +2963,9 @@
       <c r="T5" s="1">
         <v>46316</v>
       </c>
+      <c r="U5" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
@@ -2990,6 +3016,9 @@
       <c r="T6" s="1">
         <v>46316</v>
       </c>
+      <c r="U6" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
@@ -3037,6 +3066,9 @@
       <c r="R7" t="s">
         <v>38</v>
       </c>
+      <c r="U7" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W7" t="s">
         <v>55</v>
       </c>
@@ -3090,6 +3122,9 @@
       <c r="R8" t="s">
         <v>31</v>
       </c>
+      <c r="U8" s="3">
+        <v>46199</v>
+      </c>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
@@ -3140,6 +3175,9 @@
       <c r="R9" t="s">
         <v>31</v>
       </c>
+      <c r="U9" s="3">
+        <v>46244</v>
+      </c>
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
@@ -3190,6 +3228,9 @@
       <c r="T10" s="1">
         <v>46316</v>
       </c>
+      <c r="U10" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
@@ -3237,6 +3278,9 @@
       <c r="R11" t="s">
         <v>38</v>
       </c>
+      <c r="U11" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W11" t="s">
         <v>70</v>
       </c>
@@ -3290,6 +3334,9 @@
       <c r="T12" s="1">
         <v>46316</v>
       </c>
+      <c r="U12" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
@@ -3340,6 +3387,9 @@
       <c r="R13" t="s">
         <v>38</v>
       </c>
+      <c r="U13" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W13" t="s">
         <v>39</v>
       </c>
@@ -3390,6 +3440,9 @@
       <c r="R14" t="s">
         <v>38</v>
       </c>
+      <c r="U14" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W14" t="s">
         <v>55</v>
       </c>
@@ -3443,6 +3496,9 @@
       <c r="T15" s="1">
         <v>46316</v>
       </c>
+      <c r="U15" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A16" s="1">
@@ -3493,6 +3549,9 @@
       <c r="T16" s="1">
         <v>46316</v>
       </c>
+      <c r="U16" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A17" s="1">
@@ -3543,6 +3602,9 @@
       <c r="R17" t="s">
         <v>31</v>
       </c>
+      <c r="U17" s="3">
+        <v>46199</v>
+      </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A18" s="1">
@@ -3596,6 +3658,9 @@
       <c r="T18" s="1">
         <v>46316</v>
       </c>
+      <c r="U18" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A19" s="1">
@@ -3646,6 +3711,9 @@
       <c r="T19" s="1">
         <v>46316</v>
       </c>
+      <c r="U19" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A20" s="1">
@@ -3696,6 +3764,9 @@
       <c r="T20" s="1">
         <v>46316</v>
       </c>
+      <c r="U20" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A21" s="1">
@@ -3746,6 +3817,9 @@
       <c r="T21" s="1">
         <v>46316</v>
       </c>
+      <c r="U21" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A22" s="1">
@@ -3793,6 +3867,9 @@
       <c r="R22" t="s">
         <v>38</v>
       </c>
+      <c r="U22" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W22" t="s">
         <v>70</v>
       </c>
@@ -3846,6 +3923,9 @@
       <c r="T23" s="1">
         <v>46316</v>
       </c>
+      <c r="U23" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A24" s="1">
@@ -3896,6 +3976,9 @@
       <c r="R24" t="s">
         <v>38</v>
       </c>
+      <c r="U24" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W24" t="s">
         <v>39</v>
       </c>
@@ -3949,6 +4032,9 @@
       <c r="R25" t="s">
         <v>31</v>
       </c>
+      <c r="U25" s="3">
+        <v>46199</v>
+      </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A26" s="1">
@@ -3996,6 +4082,9 @@
       <c r="R26" t="s">
         <v>38</v>
       </c>
+      <c r="U26" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W26" t="s">
         <v>55</v>
       </c>
@@ -4049,6 +4138,9 @@
       <c r="R27" t="s">
         <v>38</v>
       </c>
+      <c r="U27" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W27" t="s">
         <v>39</v>
       </c>
@@ -4102,6 +4194,9 @@
       <c r="R28" t="s">
         <v>31</v>
       </c>
+      <c r="U28" s="3">
+        <v>46199</v>
+      </c>
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A29" s="1">
@@ -4149,6 +4244,9 @@
       <c r="R29" t="s">
         <v>38</v>
       </c>
+      <c r="U29" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W29" t="s">
         <v>55</v>
       </c>
@@ -4202,6 +4300,9 @@
       <c r="T30" s="1">
         <v>46316</v>
       </c>
+      <c r="U30" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A31" s="1">
@@ -4249,6 +4350,9 @@
       <c r="R31" t="s">
         <v>38</v>
       </c>
+      <c r="U31" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W31" t="s">
         <v>70</v>
       </c>
@@ -4302,6 +4406,9 @@
       <c r="R32" t="s">
         <v>31</v>
       </c>
+      <c r="U32" s="3">
+        <v>46251</v>
+      </c>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A33" s="1">
@@ -4352,6 +4459,9 @@
       <c r="R33" t="s">
         <v>31</v>
       </c>
+      <c r="U33" s="3">
+        <v>46251</v>
+      </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A34" s="1">
@@ -4399,6 +4509,9 @@
       <c r="R34" t="s">
         <v>31</v>
       </c>
+      <c r="U34" s="3">
+        <v>46266</v>
+      </c>
     </row>
     <row r="35" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A35" s="1">
@@ -4449,6 +4562,9 @@
       <c r="T35" s="1">
         <v>46316</v>
       </c>
+      <c r="U35" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="36" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A36" s="1">
@@ -4499,6 +4615,9 @@
       <c r="R36" t="s">
         <v>31</v>
       </c>
+      <c r="U36" s="3">
+        <v>46199</v>
+      </c>
     </row>
     <row r="37" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A37" s="1">
@@ -4549,6 +4668,9 @@
       <c r="R37" t="s">
         <v>31</v>
       </c>
+      <c r="U37" s="3">
+        <v>46244</v>
+      </c>
     </row>
     <row r="38" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A38" s="1">
@@ -4599,6 +4721,9 @@
       <c r="T38" s="1">
         <v>46316</v>
       </c>
+      <c r="U38" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="39" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A39" s="1">
@@ -4646,6 +4771,9 @@
       <c r="R39" t="s">
         <v>38</v>
       </c>
+      <c r="U39" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W39" t="s">
         <v>70</v>
       </c>
@@ -4696,6 +4824,9 @@
       <c r="R40" t="s">
         <v>38</v>
       </c>
+      <c r="U40" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W40" t="s">
         <v>70</v>
       </c>
@@ -4749,6 +4880,9 @@
       <c r="R41" t="s">
         <v>38</v>
       </c>
+      <c r="U41" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W41" t="s">
         <v>39</v>
       </c>
@@ -4799,6 +4933,9 @@
       <c r="R42" t="s">
         <v>38</v>
       </c>
+      <c r="U42" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W42" t="s">
         <v>55</v>
       </c>
@@ -4855,6 +4992,9 @@
       <c r="T43" s="1">
         <v>46316</v>
       </c>
+      <c r="U43" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A44" s="1">
@@ -4905,6 +5045,9 @@
       <c r="T44" s="1">
         <v>46316</v>
       </c>
+      <c r="U44" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="45" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A45" s="1">
@@ -4955,6 +5098,9 @@
       <c r="T45" s="1">
         <v>46316</v>
       </c>
+      <c r="U45" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="46" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A46" s="1">
@@ -5005,6 +5151,9 @@
       <c r="R46" t="s">
         <v>38</v>
       </c>
+      <c r="U46" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W46" t="s">
         <v>39</v>
       </c>
@@ -5058,6 +5207,9 @@
       <c r="R47" t="s">
         <v>31</v>
       </c>
+      <c r="U47" s="3">
+        <v>46244</v>
+      </c>
     </row>
     <row r="48" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A48" s="1">
@@ -5108,6 +5260,9 @@
       <c r="R48" t="s">
         <v>31</v>
       </c>
+      <c r="U48" s="3">
+        <v>46199</v>
+      </c>
     </row>
     <row r="49" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A49" s="1">
@@ -5158,6 +5313,9 @@
       <c r="R49" t="s">
         <v>31</v>
       </c>
+      <c r="U49" s="3">
+        <v>46244</v>
+      </c>
     </row>
     <row r="50" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A50" s="1">
@@ -5208,6 +5366,9 @@
       <c r="R50" t="s">
         <v>31</v>
       </c>
+      <c r="U50" s="3">
+        <v>46251</v>
+      </c>
     </row>
     <row r="51" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A51" s="1">
@@ -5258,6 +5419,9 @@
       <c r="R51" t="s">
         <v>31</v>
       </c>
+      <c r="U51" s="3">
+        <v>46199</v>
+      </c>
     </row>
     <row r="52" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A52" s="1">
@@ -5305,6 +5469,9 @@
       <c r="R52" t="s">
         <v>38</v>
       </c>
+      <c r="U52" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W52" t="s">
         <v>55</v>
       </c>
@@ -5358,6 +5525,9 @@
       <c r="R53" t="s">
         <v>31</v>
       </c>
+      <c r="U53" s="3">
+        <v>46244</v>
+      </c>
     </row>
     <row r="54" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A54" s="1">
@@ -5408,6 +5578,9 @@
       <c r="R54" t="s">
         <v>38</v>
       </c>
+      <c r="U54" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W54" t="s">
         <v>39</v>
       </c>
@@ -5458,6 +5631,9 @@
       <c r="R55" t="s">
         <v>31</v>
       </c>
+      <c r="U55" s="3">
+        <v>46199</v>
+      </c>
     </row>
     <row r="56" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A56" s="1">
@@ -5508,6 +5684,9 @@
       <c r="R56" t="s">
         <v>38</v>
       </c>
+      <c r="U56" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W56" t="s">
         <v>39</v>
       </c>
@@ -5561,6 +5740,9 @@
       <c r="R57" t="s">
         <v>31</v>
       </c>
+      <c r="U57" s="3">
+        <v>46199</v>
+      </c>
     </row>
     <row r="58" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A58" s="1">
@@ -5608,6 +5790,9 @@
       <c r="R58" t="s">
         <v>38</v>
       </c>
+      <c r="U58" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W58" t="s">
         <v>207</v>
       </c>
@@ -5658,6 +5843,9 @@
       <c r="R59" t="s">
         <v>38</v>
       </c>
+      <c r="U59" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W59" t="s">
         <v>207</v>
       </c>
@@ -5711,6 +5899,9 @@
       <c r="R60" t="s">
         <v>38</v>
       </c>
+      <c r="U60" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W60" t="s">
         <v>39</v>
       </c>
@@ -5761,6 +5952,9 @@
       <c r="R61" t="s">
         <v>38</v>
       </c>
+      <c r="U61" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W61" t="s">
         <v>70</v>
       </c>
@@ -5814,6 +6008,9 @@
       <c r="R62" t="s">
         <v>31</v>
       </c>
+      <c r="U62" s="3">
+        <v>46199</v>
+      </c>
     </row>
     <row r="63" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A63" s="1">
@@ -5867,6 +6064,9 @@
       <c r="T63" s="1">
         <v>46316</v>
       </c>
+      <c r="U63" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="64" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A64" s="1">
@@ -5920,6 +6120,9 @@
       <c r="T64" s="1">
         <v>46316</v>
       </c>
+      <c r="U64" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="65" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A65" s="1">
@@ -5967,6 +6170,9 @@
       <c r="R65" t="s">
         <v>38</v>
       </c>
+      <c r="U65" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W65" t="s">
         <v>70</v>
       </c>
@@ -6020,6 +6226,9 @@
       <c r="R66" t="s">
         <v>38</v>
       </c>
+      <c r="U66" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W66" t="s">
         <v>39</v>
       </c>
@@ -6073,6 +6282,9 @@
       <c r="R67" t="s">
         <v>38</v>
       </c>
+      <c r="U67" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W67" t="s">
         <v>39</v>
       </c>
@@ -6126,6 +6338,9 @@
       <c r="R68" t="s">
         <v>31</v>
       </c>
+      <c r="U68" s="3">
+        <v>46244</v>
+      </c>
     </row>
     <row r="69" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A69" s="1">
@@ -6179,6 +6394,9 @@
       <c r="R69" t="s">
         <v>31</v>
       </c>
+      <c r="U69" s="3">
+        <v>46199</v>
+      </c>
     </row>
     <row r="70" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A70" s="1">
@@ -6226,6 +6444,9 @@
       <c r="R70" t="s">
         <v>38</v>
       </c>
+      <c r="U70" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W70" t="s">
         <v>70</v>
       </c>
@@ -6285,6 +6506,9 @@
       <c r="T71" s="1">
         <v>46316</v>
       </c>
+      <c r="U71" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="72" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A72" s="1">
@@ -6335,6 +6559,9 @@
       <c r="T72" s="1">
         <v>46316</v>
       </c>
+      <c r="U72" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="73" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A73" s="1">
@@ -6385,6 +6612,9 @@
       <c r="R73" t="s">
         <v>31</v>
       </c>
+      <c r="U73" s="3">
+        <v>46199</v>
+      </c>
     </row>
     <row r="74" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A74" s="1">
@@ -6432,6 +6662,9 @@
       <c r="R74" t="s">
         <v>38</v>
       </c>
+      <c r="U74" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W74" t="s">
         <v>55</v>
       </c>
@@ -6482,6 +6715,9 @@
       <c r="R75" t="s">
         <v>31</v>
       </c>
+      <c r="U75" s="3">
+        <v>46244</v>
+      </c>
     </row>
     <row r="76" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A76" s="1">
@@ -6532,6 +6768,9 @@
       <c r="R76" t="s">
         <v>31</v>
       </c>
+      <c r="U76" s="3">
+        <v>46258</v>
+      </c>
     </row>
     <row r="77" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A77" s="1">
@@ -6579,6 +6818,9 @@
       <c r="R77" t="s">
         <v>38</v>
       </c>
+      <c r="U77" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W77" t="s">
         <v>70</v>
       </c>
@@ -6629,6 +6871,9 @@
       <c r="R78" t="s">
         <v>38</v>
       </c>
+      <c r="U78" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W78" t="s">
         <v>70</v>
       </c>
@@ -6679,6 +6924,9 @@
       <c r="R79" t="s">
         <v>38</v>
       </c>
+      <c r="U79" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W79" t="s">
         <v>70</v>
       </c>
@@ -6729,6 +6977,9 @@
       <c r="R80" t="s">
         <v>38</v>
       </c>
+      <c r="U80" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W80" t="s">
         <v>70</v>
       </c>
@@ -6782,6 +7033,9 @@
       <c r="T81" s="1">
         <v>46316</v>
       </c>
+      <c r="U81" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="82" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A82" s="1">
@@ -6829,6 +7083,9 @@
       <c r="R82" t="s">
         <v>31</v>
       </c>
+      <c r="U82" s="3">
+        <v>46199</v>
+      </c>
     </row>
     <row r="83" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A83" s="1">
@@ -6876,6 +7133,9 @@
       <c r="R83" t="s">
         <v>38</v>
       </c>
+      <c r="U83" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W83" t="s">
         <v>70</v>
       </c>
@@ -6935,6 +7195,9 @@
       <c r="T84" s="1">
         <v>46316</v>
       </c>
+      <c r="U84" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="85" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A85" s="1">
@@ -6985,6 +7248,9 @@
       <c r="T85" s="1">
         <v>46316</v>
       </c>
+      <c r="U85" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="86" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A86" s="1">
@@ -7035,6 +7301,9 @@
       <c r="R86" t="s">
         <v>31</v>
       </c>
+      <c r="U86" s="3">
+        <v>46266</v>
+      </c>
     </row>
     <row r="87" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A87" s="1">
@@ -7085,6 +7354,9 @@
       <c r="T87" s="1">
         <v>46316</v>
       </c>
+      <c r="U87" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="88" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A88" s="1">
@@ -7135,6 +7407,9 @@
       <c r="T88" s="1">
         <v>46316</v>
       </c>
+      <c r="U88" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="89" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A89" s="1">
@@ -7182,6 +7457,9 @@
       <c r="R89" t="s">
         <v>31</v>
       </c>
+      <c r="U89" s="3">
+        <v>46199</v>
+      </c>
     </row>
     <row r="90" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A90" s="1">
@@ -7229,6 +7507,9 @@
       <c r="R90" t="s">
         <v>38</v>
       </c>
+      <c r="U90" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W90" t="s">
         <v>70</v>
       </c>
@@ -7282,6 +7563,9 @@
       <c r="R91" t="s">
         <v>31</v>
       </c>
+      <c r="U91" s="3">
+        <v>46251</v>
+      </c>
     </row>
     <row r="92" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A92" s="1">
@@ -7329,6 +7613,9 @@
       <c r="R92" t="s">
         <v>38</v>
       </c>
+      <c r="U92" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W92" t="s">
         <v>55</v>
       </c>
@@ -7379,6 +7666,9 @@
       <c r="R93" t="s">
         <v>38</v>
       </c>
+      <c r="U93" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W93" t="s">
         <v>70</v>
       </c>
@@ -7435,6 +7725,9 @@
       <c r="T94" s="1">
         <v>46316</v>
       </c>
+      <c r="U94" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="95" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A95" s="1">
@@ -7482,6 +7775,9 @@
       <c r="R95" t="s">
         <v>38</v>
       </c>
+      <c r="U95" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W95" t="s">
         <v>70</v>
       </c>
@@ -7532,6 +7828,9 @@
       <c r="R96" t="s">
         <v>38</v>
       </c>
+      <c r="U96" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W96" t="s">
         <v>70</v>
       </c>
@@ -7585,6 +7884,9 @@
       <c r="R97" t="s">
         <v>38</v>
       </c>
+      <c r="U97" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W97" t="s">
         <v>39</v>
       </c>
@@ -7635,6 +7937,9 @@
       <c r="R98" t="s">
         <v>38</v>
       </c>
+      <c r="U98" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W98" t="s">
         <v>55</v>
       </c>
@@ -7685,6 +7990,9 @@
       <c r="R99" t="s">
         <v>31</v>
       </c>
+      <c r="U99" s="3">
+        <v>46258</v>
+      </c>
     </row>
     <row r="100" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A100" s="1">
@@ -7732,6 +8040,9 @@
       <c r="R100" t="s">
         <v>38</v>
       </c>
+      <c r="U100" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W100" t="s">
         <v>70</v>
       </c>
@@ -7782,6 +8093,9 @@
       <c r="R101" t="s">
         <v>38</v>
       </c>
+      <c r="U101" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W101" t="s">
         <v>55</v>
       </c>
@@ -7835,6 +8149,9 @@
       <c r="T102" s="1">
         <v>46316</v>
       </c>
+      <c r="U102" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="103" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A103" s="1">
@@ -7885,6 +8202,9 @@
       <c r="R103" t="s">
         <v>31</v>
       </c>
+      <c r="U103" s="3">
+        <v>46244</v>
+      </c>
     </row>
     <row r="104" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A104" s="1">
@@ -7932,6 +8252,9 @@
       <c r="R104" t="s">
         <v>38</v>
       </c>
+      <c r="U104" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W104" t="s">
         <v>55</v>
       </c>
@@ -7982,6 +8305,9 @@
       <c r="R105" t="s">
         <v>38</v>
       </c>
+      <c r="U105" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W105" t="s">
         <v>70</v>
       </c>
@@ -8035,6 +8361,9 @@
       <c r="R106" t="s">
         <v>31</v>
       </c>
+      <c r="U106" s="3">
+        <v>46251</v>
+      </c>
     </row>
     <row r="107" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A107" s="1">
@@ -8085,6 +8414,9 @@
       <c r="R107" t="s">
         <v>38</v>
       </c>
+      <c r="U107" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W107" t="s">
         <v>39</v>
       </c>
@@ -8141,6 +8473,9 @@
       <c r="T108" s="1">
         <v>46316</v>
       </c>
+      <c r="U108" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="109" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A109" s="1">
@@ -8191,6 +8526,9 @@
       <c r="T109" s="1">
         <v>46316</v>
       </c>
+      <c r="U109" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="110" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A110" s="1">
@@ -8238,6 +8576,9 @@
       <c r="R110" t="s">
         <v>38</v>
       </c>
+      <c r="U110" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W110" t="s">
         <v>55</v>
       </c>
@@ -8288,6 +8629,9 @@
       <c r="R111" t="s">
         <v>38</v>
       </c>
+      <c r="U111" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W111" t="s">
         <v>70</v>
       </c>
@@ -8341,6 +8685,9 @@
       <c r="R112" t="s">
         <v>38</v>
       </c>
+      <c r="U112" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W112" t="s">
         <v>39</v>
       </c>
@@ -8394,6 +8741,9 @@
       <c r="R113" t="s">
         <v>31</v>
       </c>
+      <c r="U113" s="3">
+        <v>46244</v>
+      </c>
     </row>
     <row r="114" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A114" s="1">
@@ -8444,6 +8794,9 @@
       <c r="R114" t="s">
         <v>31</v>
       </c>
+      <c r="U114" s="3">
+        <v>46199</v>
+      </c>
     </row>
     <row r="115" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A115" s="1">
@@ -8494,6 +8847,9 @@
       <c r="R115" t="s">
         <v>31</v>
       </c>
+      <c r="U115" s="3">
+        <v>46244</v>
+      </c>
     </row>
     <row r="116" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A116" s="1">
@@ -8541,6 +8897,9 @@
       <c r="R116" t="s">
         <v>38</v>
       </c>
+      <c r="U116" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W116" t="s">
         <v>70</v>
       </c>
@@ -8591,6 +8950,9 @@
       <c r="R117" t="s">
         <v>38</v>
       </c>
+      <c r="U117" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W117" t="s">
         <v>70</v>
       </c>
@@ -8641,6 +9003,9 @@
       <c r="R118" t="s">
         <v>38</v>
       </c>
+      <c r="U118" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W118" t="s">
         <v>55</v>
       </c>
@@ -8694,6 +9059,9 @@
       <c r="T119" s="1">
         <v>46316</v>
       </c>
+      <c r="U119" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="120" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A120" s="1">
@@ -8744,6 +9112,9 @@
       <c r="T120" s="1">
         <v>46316</v>
       </c>
+      <c r="U120" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="121" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A121" s="1">
@@ -8791,6 +9162,9 @@
       <c r="R121" t="s">
         <v>38</v>
       </c>
+      <c r="U121" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W121" t="s">
         <v>70</v>
       </c>
@@ -8841,6 +9215,9 @@
       <c r="R122" t="s">
         <v>38</v>
       </c>
+      <c r="U122" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W122" t="s">
         <v>70</v>
       </c>
@@ -8894,6 +9271,9 @@
       <c r="R123" t="s">
         <v>38</v>
       </c>
+      <c r="U123" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W123" t="s">
         <v>39</v>
       </c>
@@ -8944,6 +9324,9 @@
       <c r="R124" t="s">
         <v>38</v>
       </c>
+      <c r="U124" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W124" t="s">
         <v>55</v>
       </c>
@@ -8997,6 +9380,9 @@
       <c r="R125" t="s">
         <v>31</v>
       </c>
+      <c r="U125" s="3">
+        <v>46216</v>
+      </c>
     </row>
     <row r="126" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A126" s="1">
@@ -9047,6 +9433,9 @@
       <c r="T126" s="1">
         <v>46316</v>
       </c>
+      <c r="U126" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="127" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A127" s="1">
@@ -9094,6 +9483,9 @@
       <c r="R127" t="s">
         <v>38</v>
       </c>
+      <c r="U127" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W127" t="s">
         <v>70</v>
       </c>
@@ -9144,6 +9536,9 @@
       <c r="R128" t="s">
         <v>38</v>
       </c>
+      <c r="U128" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W128" t="s">
         <v>70</v>
       </c>
@@ -9194,6 +9589,9 @@
       <c r="R129" t="s">
         <v>38</v>
       </c>
+      <c r="U129" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W129" t="s">
         <v>55</v>
       </c>
@@ -9247,6 +9645,9 @@
       <c r="R130" t="s">
         <v>38</v>
       </c>
+      <c r="U130" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W130" t="s">
         <v>39</v>
       </c>
@@ -9297,6 +9698,9 @@
       <c r="R131" t="s">
         <v>38</v>
       </c>
+      <c r="U131" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W131" t="s">
         <v>55</v>
       </c>
@@ -9350,6 +9754,9 @@
       <c r="R132" t="s">
         <v>31</v>
       </c>
+      <c r="U132" s="3">
+        <v>46244</v>
+      </c>
     </row>
     <row r="133" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A133" s="1">
@@ -9397,6 +9804,9 @@
       <c r="R133" t="s">
         <v>38</v>
       </c>
+      <c r="U133" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W133" t="s">
         <v>70</v>
       </c>
@@ -9447,6 +9857,9 @@
       <c r="R134" t="s">
         <v>38</v>
       </c>
+      <c r="U134" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W134" t="s">
         <v>70</v>
       </c>
@@ -9497,6 +9910,9 @@
       <c r="R135" t="s">
         <v>38</v>
       </c>
+      <c r="U135" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W135" t="s">
         <v>70</v>
       </c>
@@ -9553,6 +9969,9 @@
       <c r="T136" s="1">
         <v>46316</v>
       </c>
+      <c r="U136" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="137" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A137" s="1">
@@ -9603,6 +10022,9 @@
       <c r="T137" s="1">
         <v>46316</v>
       </c>
+      <c r="U137" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="138" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A138" s="1">
@@ -9653,6 +10075,9 @@
       <c r="T138" s="1">
         <v>46316</v>
       </c>
+      <c r="U138" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="139" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A139" s="1">
@@ -9700,6 +10125,9 @@
       <c r="R139" t="s">
         <v>38</v>
       </c>
+      <c r="U139" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W139" t="s">
         <v>55</v>
       </c>
@@ -9753,6 +10181,9 @@
       <c r="T140" s="1">
         <v>46316</v>
       </c>
+      <c r="U140" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="141" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A141" s="1">
@@ -9800,6 +10231,9 @@
       <c r="R141" t="s">
         <v>38</v>
       </c>
+      <c r="U141" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W141" t="s">
         <v>70</v>
       </c>
@@ -9853,6 +10287,9 @@
       <c r="R142" t="s">
         <v>31</v>
       </c>
+      <c r="U142" s="3">
+        <v>46216</v>
+      </c>
     </row>
     <row r="143" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A143" s="1">
@@ -9900,6 +10337,9 @@
       <c r="R143" t="s">
         <v>38</v>
       </c>
+      <c r="U143" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W143" t="s">
         <v>70</v>
       </c>
@@ -9953,6 +10393,9 @@
       <c r="R144" t="s">
         <v>31</v>
       </c>
+      <c r="U144" s="3">
+        <v>46251</v>
+      </c>
     </row>
     <row r="145" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A145" s="1">
@@ -10000,6 +10443,9 @@
       <c r="R145" t="s">
         <v>38</v>
       </c>
+      <c r="U145" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W145" t="s">
         <v>70</v>
       </c>
@@ -10047,6 +10493,9 @@
       <c r="R146" t="s">
         <v>38</v>
       </c>
+      <c r="U146" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W146" t="s">
         <v>70</v>
       </c>
@@ -10094,6 +10543,9 @@
       <c r="R147" t="s">
         <v>38</v>
       </c>
+      <c r="U147" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W147" t="s">
         <v>55</v>
       </c>
@@ -10141,6 +10593,9 @@
       <c r="R148" t="s">
         <v>38</v>
       </c>
+      <c r="U148" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W148" t="s">
         <v>70</v>
       </c>
@@ -10182,6 +10637,9 @@
       <c r="R149" t="s">
         <v>38</v>
       </c>
+      <c r="U149" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W149" t="s">
         <v>207</v>
       </c>
@@ -10223,6 +10681,9 @@
       <c r="R150" t="s">
         <v>38</v>
       </c>
+      <c r="U150" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W150" t="s">
         <v>207</v>
       </c>
@@ -10264,6 +10725,9 @@
       <c r="R151" t="s">
         <v>38</v>
       </c>
+      <c r="U151" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W151" t="s">
         <v>207</v>
       </c>
@@ -10305,6 +10769,9 @@
       <c r="R152" t="s">
         <v>38</v>
       </c>
+      <c r="U152" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W152" t="s">
         <v>207</v>
       </c>
@@ -10346,6 +10813,9 @@
       <c r="R153" t="s">
         <v>38</v>
       </c>
+      <c r="U153" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W153" t="s">
         <v>207</v>
       </c>
@@ -10387,6 +10857,9 @@
       <c r="R154" t="s">
         <v>38</v>
       </c>
+      <c r="U154" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W154" t="s">
         <v>207</v>
       </c>
@@ -10428,6 +10901,9 @@
       <c r="R155" t="s">
         <v>38</v>
       </c>
+      <c r="U155" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W155" t="s">
         <v>207</v>
       </c>
@@ -10469,6 +10945,9 @@
       <c r="R156" t="s">
         <v>38</v>
       </c>
+      <c r="U156" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W156" t="s">
         <v>207</v>
       </c>
@@ -10516,6 +10995,9 @@
       <c r="T157" s="1">
         <v>46316</v>
       </c>
+      <c r="U157" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="158" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A158" s="1">
@@ -10554,6 +11036,9 @@
       <c r="R158" t="s">
         <v>38</v>
       </c>
+      <c r="U158" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W158" t="s">
         <v>207</v>
       </c>
@@ -10595,6 +11080,9 @@
       <c r="R159" t="s">
         <v>38</v>
       </c>
+      <c r="U159" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W159" t="s">
         <v>207</v>
       </c>
@@ -10636,6 +11124,9 @@
       <c r="R160" t="s">
         <v>38</v>
       </c>
+      <c r="U160" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W160" t="s">
         <v>207</v>
       </c>
@@ -10683,6 +11174,9 @@
       <c r="T161" s="1">
         <v>46316</v>
       </c>
+      <c r="U161" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="162" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A162" s="1">
@@ -10721,6 +11215,9 @@
       <c r="R162" t="s">
         <v>38</v>
       </c>
+      <c r="U162" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W162" t="s">
         <v>207</v>
       </c>
@@ -10768,6 +11265,9 @@
       <c r="R163" t="s">
         <v>38</v>
       </c>
+      <c r="U163" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W163" t="s">
         <v>70</v>
       </c>
@@ -10809,6 +11309,9 @@
       <c r="R164" t="s">
         <v>38</v>
       </c>
+      <c r="U164" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W164" t="s">
         <v>207</v>
       </c>
@@ -10850,6 +11353,9 @@
       <c r="R165" t="s">
         <v>38</v>
       </c>
+      <c r="U165" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W165" t="s">
         <v>207</v>
       </c>
@@ -10897,6 +11403,9 @@
       <c r="T166" s="1">
         <v>46316</v>
       </c>
+      <c r="U166" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="167" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A167" s="1">
@@ -10935,6 +11444,9 @@
       <c r="R167" t="s">
         <v>38</v>
       </c>
+      <c r="U167" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W167" t="s">
         <v>207</v>
       </c>
@@ -10982,6 +11494,9 @@
       <c r="T168" s="1">
         <v>46316</v>
       </c>
+      <c r="U168" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="169" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A169" s="1">
@@ -11020,6 +11535,9 @@
       <c r="R169" t="s">
         <v>38</v>
       </c>
+      <c r="U169" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W169" t="s">
         <v>207</v>
       </c>
@@ -11061,6 +11579,9 @@
       <c r="R170" t="s">
         <v>38</v>
       </c>
+      <c r="U170" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W170" t="s">
         <v>207</v>
       </c>
@@ -11108,6 +11629,9 @@
       <c r="T171" s="1">
         <v>46316</v>
       </c>
+      <c r="U171" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="172" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A172" s="1">
@@ -11146,6 +11670,9 @@
       <c r="R172" t="s">
         <v>38</v>
       </c>
+      <c r="U172" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W172" t="s">
         <v>207</v>
       </c>
@@ -11187,6 +11714,9 @@
       <c r="R173" t="s">
         <v>38</v>
       </c>
+      <c r="U173" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W173" t="s">
         <v>207</v>
       </c>
@@ -11234,6 +11764,9 @@
       <c r="T174" s="1">
         <v>46316</v>
       </c>
+      <c r="U174" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="175" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A175" s="1">
@@ -11272,6 +11805,9 @@
       <c r="R175" t="s">
         <v>38</v>
       </c>
+      <c r="U175" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W175" t="s">
         <v>207</v>
       </c>
@@ -11319,6 +11855,9 @@
       <c r="T176" s="1">
         <v>46316</v>
       </c>
+      <c r="U176" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="177" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A177" s="1">
@@ -11357,6 +11896,9 @@
       <c r="R177" t="s">
         <v>38</v>
       </c>
+      <c r="U177" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W177" t="s">
         <v>207</v>
       </c>
@@ -11404,6 +11946,9 @@
       <c r="T178" s="1">
         <v>46316</v>
       </c>
+      <c r="U178" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="179" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A179" s="1">
@@ -11448,6 +11993,9 @@
       <c r="T179" s="1">
         <v>46316</v>
       </c>
+      <c r="U179" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="180" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A180" s="1">
@@ -11498,6 +12046,9 @@
       <c r="T180" s="1">
         <v>46316</v>
       </c>
+      <c r="U180" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="181" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A181" s="1">
@@ -11539,6 +12090,9 @@
       <c r="R181" t="s">
         <v>38</v>
       </c>
+      <c r="U181" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W181" t="s">
         <v>207</v>
       </c>
@@ -11580,6 +12134,9 @@
       <c r="R182" t="s">
         <v>38</v>
       </c>
+      <c r="U182" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W182" t="s">
         <v>207</v>
       </c>
@@ -11627,6 +12184,9 @@
       <c r="T183" s="1">
         <v>46316</v>
       </c>
+      <c r="U183" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="184" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A184" s="1">
@@ -11665,6 +12225,9 @@
       <c r="R184" t="s">
         <v>38</v>
       </c>
+      <c r="U184" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W184" t="s">
         <v>207</v>
       </c>
@@ -11706,6 +12269,9 @@
       <c r="R185" t="s">
         <v>38</v>
       </c>
+      <c r="U185" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W185" t="s">
         <v>207</v>
       </c>
@@ -11747,6 +12313,9 @@
       <c r="R186" t="s">
         <v>38</v>
       </c>
+      <c r="U186" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W186" t="s">
         <v>207</v>
       </c>
@@ -11788,6 +12357,9 @@
       <c r="R187" t="s">
         <v>38</v>
       </c>
+      <c r="U187" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W187" t="s">
         <v>207</v>
       </c>
@@ -11829,6 +12401,9 @@
       <c r="R188" t="s">
         <v>38</v>
       </c>
+      <c r="U188" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W188" t="s">
         <v>207</v>
       </c>
@@ -11870,6 +12445,9 @@
       <c r="R189" t="s">
         <v>38</v>
       </c>
+      <c r="U189" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W189" t="s">
         <v>207</v>
       </c>
@@ -11917,6 +12495,9 @@
       <c r="T190" s="1">
         <v>46316</v>
       </c>
+      <c r="U190" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="191" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A191" s="1">
@@ -11955,6 +12536,9 @@
       <c r="R191" t="s">
         <v>38</v>
       </c>
+      <c r="U191" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W191" t="s">
         <v>207</v>
       </c>
@@ -12002,6 +12586,9 @@
       <c r="R192" t="s">
         <v>38</v>
       </c>
+      <c r="U192" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W192" t="s">
         <v>70</v>
       </c>
@@ -12043,6 +12630,9 @@
       <c r="R193" t="s">
         <v>38</v>
       </c>
+      <c r="U193" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W193" t="s">
         <v>207</v>
       </c>
@@ -12084,6 +12674,9 @@
       <c r="R194" t="s">
         <v>38</v>
       </c>
+      <c r="U194" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W194" t="s">
         <v>207</v>
       </c>
@@ -12125,6 +12718,9 @@
       <c r="R195" t="s">
         <v>38</v>
       </c>
+      <c r="U195" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W195" t="s">
         <v>207</v>
       </c>
@@ -12166,6 +12762,9 @@
       <c r="R196" t="s">
         <v>38</v>
       </c>
+      <c r="U196" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W196" t="s">
         <v>207</v>
       </c>
@@ -12207,6 +12806,9 @@
       <c r="R197" t="s">
         <v>38</v>
       </c>
+      <c r="U197" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W197" t="s">
         <v>207</v>
       </c>
@@ -12248,6 +12850,9 @@
       <c r="R198" t="s">
         <v>38</v>
       </c>
+      <c r="U198" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W198" t="s">
         <v>207</v>
       </c>
@@ -12289,6 +12894,9 @@
       <c r="R199" t="s">
         <v>38</v>
       </c>
+      <c r="U199" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W199" t="s">
         <v>207</v>
       </c>
@@ -12330,6 +12938,9 @@
       <c r="R200" t="s">
         <v>38</v>
       </c>
+      <c r="U200" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W200" t="s">
         <v>207</v>
       </c>
@@ -12377,6 +12988,9 @@
       <c r="T201" s="1">
         <v>46316</v>
       </c>
+      <c r="U201" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="202" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A202" s="1">
@@ -12421,6 +13035,9 @@
       <c r="T202" s="1">
         <v>46316</v>
       </c>
+      <c r="U202" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="203" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A203" s="1">
@@ -12465,6 +13082,9 @@
       <c r="T203" s="1">
         <v>46316</v>
       </c>
+      <c r="U203" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="204" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A204" s="1">
@@ -12509,6 +13129,9 @@
       <c r="T204" s="1">
         <v>46316</v>
       </c>
+      <c r="U204" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="205" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A205" s="1">
@@ -12547,6 +13170,9 @@
       <c r="R205" t="s">
         <v>38</v>
       </c>
+      <c r="U205" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W205" t="s">
         <v>207</v>
       </c>
@@ -12594,6 +13220,9 @@
       <c r="T206" s="1">
         <v>46316</v>
       </c>
+      <c r="U206" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="207" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A207" s="1">
@@ -12632,6 +13261,9 @@
       <c r="R207" t="s">
         <v>38</v>
       </c>
+      <c r="U207" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W207" t="s">
         <v>207</v>
       </c>
@@ -12679,6 +13311,9 @@
       <c r="T208" s="1">
         <v>46316</v>
       </c>
+      <c r="U208" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="209" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A209" s="1">
@@ -12717,6 +13352,9 @@
       <c r="R209" t="s">
         <v>38</v>
       </c>
+      <c r="U209" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W209" t="s">
         <v>207</v>
       </c>
@@ -12764,6 +13402,9 @@
       <c r="T210" s="1">
         <v>46316</v>
       </c>
+      <c r="U210" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="211" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A211" s="1">
@@ -12808,6 +13449,9 @@
       <c r="T211" s="1">
         <v>46316</v>
       </c>
+      <c r="U211" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="212" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A212" s="1">
@@ -12852,6 +13496,9 @@
       <c r="T212" s="1">
         <v>46316</v>
       </c>
+      <c r="U212" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="213" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A213" s="1">
@@ -12890,6 +13537,9 @@
       <c r="R213" t="s">
         <v>38</v>
       </c>
+      <c r="U213" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W213" t="s">
         <v>207</v>
       </c>
@@ -12937,6 +13587,9 @@
       <c r="T214" s="1">
         <v>46316</v>
       </c>
+      <c r="U214" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="215" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A215" s="1">
@@ -12981,6 +13634,9 @@
       <c r="T215" s="1">
         <v>46316</v>
       </c>
+      <c r="U215" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="216" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A216" s="1">
@@ -13019,6 +13675,9 @@
       <c r="R216" t="s">
         <v>38</v>
       </c>
+      <c r="U216" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W216" t="s">
         <v>207</v>
       </c>
@@ -13060,6 +13719,9 @@
       <c r="R217" t="s">
         <v>38</v>
       </c>
+      <c r="U217" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W217" t="s">
         <v>207</v>
       </c>
@@ -13101,6 +13763,9 @@
       <c r="R218" t="s">
         <v>38</v>
       </c>
+      <c r="U218" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W218" t="s">
         <v>207</v>
       </c>
@@ -13148,6 +13813,9 @@
       <c r="T219" s="1">
         <v>46316</v>
       </c>
+      <c r="U219" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="220" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A220" s="1">
@@ -13186,6 +13854,9 @@
       <c r="R220" t="s">
         <v>38</v>
       </c>
+      <c r="U220" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W220" t="s">
         <v>207</v>
       </c>
@@ -13227,6 +13898,9 @@
       <c r="R221" t="s">
         <v>38</v>
       </c>
+      <c r="U221" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W221" t="s">
         <v>207</v>
       </c>
@@ -13274,6 +13948,9 @@
       <c r="T222" s="1">
         <v>46316</v>
       </c>
+      <c r="U222" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="223" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A223" s="1">
@@ -13312,6 +13989,9 @@
       <c r="R223" t="s">
         <v>38</v>
       </c>
+      <c r="U223" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W223" t="s">
         <v>207</v>
       </c>
@@ -13359,6 +14039,9 @@
       <c r="T224" s="1">
         <v>46316</v>
       </c>
+      <c r="U224" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="225" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A225" s="1">
@@ -13397,6 +14080,9 @@
       <c r="R225" t="s">
         <v>38</v>
       </c>
+      <c r="U225" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W225" t="s">
         <v>207</v>
       </c>
@@ -13438,6 +14124,9 @@
       <c r="R226" t="s">
         <v>38</v>
       </c>
+      <c r="U226" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W226" t="s">
         <v>207</v>
       </c>
@@ -13479,6 +14168,9 @@
       <c r="R227" t="s">
         <v>38</v>
       </c>
+      <c r="U227" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W227" t="s">
         <v>207</v>
       </c>
@@ -13520,6 +14212,9 @@
       <c r="R228" t="s">
         <v>38</v>
       </c>
+      <c r="U228" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W228" t="s">
         <v>207</v>
       </c>
@@ -13561,6 +14256,9 @@
       <c r="R229" t="s">
         <v>38</v>
       </c>
+      <c r="U229" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W229" t="s">
         <v>207</v>
       </c>
@@ -13602,6 +14300,9 @@
       <c r="R230" t="s">
         <v>38</v>
       </c>
+      <c r="U230" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W230" t="s">
         <v>207</v>
       </c>
@@ -13643,6 +14344,9 @@
       <c r="R231" t="s">
         <v>38</v>
       </c>
+      <c r="U231" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W231" t="s">
         <v>207</v>
       </c>
@@ -13690,6 +14394,9 @@
       <c r="T232" s="1">
         <v>46316</v>
       </c>
+      <c r="U232" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="233" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A233" s="1">
@@ -13734,6 +14441,9 @@
       <c r="T233" s="1">
         <v>46316</v>
       </c>
+      <c r="U233" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="234" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A234" s="1">
@@ -13772,6 +14482,9 @@
       <c r="R234" t="s">
         <v>38</v>
       </c>
+      <c r="U234" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W234" t="s">
         <v>207</v>
       </c>
@@ -13813,6 +14526,9 @@
       <c r="R235" t="s">
         <v>38</v>
       </c>
+      <c r="U235" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W235" t="s">
         <v>207</v>
       </c>
@@ -13854,6 +14570,9 @@
       <c r="R236" t="s">
         <v>38</v>
       </c>
+      <c r="U236" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W236" t="s">
         <v>207</v>
       </c>
@@ -13895,6 +14614,9 @@
       <c r="R237" t="s">
         <v>38</v>
       </c>
+      <c r="U237" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W237" t="s">
         <v>207</v>
       </c>
@@ -13936,6 +14658,9 @@
       <c r="R238" t="s">
         <v>38</v>
       </c>
+      <c r="U238" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W238" t="s">
         <v>207</v>
       </c>
@@ -13983,6 +14708,9 @@
       <c r="T239" s="1">
         <v>46316</v>
       </c>
+      <c r="U239" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="240" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A240" s="1">
@@ -14027,6 +14755,9 @@
       <c r="T240" s="1">
         <v>46316</v>
       </c>
+      <c r="U240" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="241" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A241" s="1">
@@ -14065,6 +14796,9 @@
       <c r="R241" t="s">
         <v>38</v>
       </c>
+      <c r="U241" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W241" t="s">
         <v>207</v>
       </c>
@@ -14106,6 +14840,9 @@
       <c r="R242" t="s">
         <v>38</v>
       </c>
+      <c r="U242" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W242" t="s">
         <v>207</v>
       </c>
@@ -14147,6 +14884,9 @@
       <c r="R243" t="s">
         <v>38</v>
       </c>
+      <c r="U243" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W243" t="s">
         <v>207</v>
       </c>
@@ -14188,6 +14928,9 @@
       <c r="R244" t="s">
         <v>38</v>
       </c>
+      <c r="U244" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W244" t="s">
         <v>207</v>
       </c>
@@ -14229,6 +14972,9 @@
       <c r="R245" t="s">
         <v>38</v>
       </c>
+      <c r="U245" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W245" t="s">
         <v>207</v>
       </c>
@@ -14270,6 +15016,9 @@
       <c r="R246" t="s">
         <v>38</v>
       </c>
+      <c r="U246" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W246" t="s">
         <v>207</v>
       </c>
@@ -14311,6 +15060,9 @@
       <c r="R247" t="s">
         <v>38</v>
       </c>
+      <c r="U247" s="3" t="s">
+        <v>696</v>
+      </c>
       <c r="W247" t="s">
         <v>207</v>
       </c>
@@ -14358,6 +15110,9 @@
       <c r="T248" s="1">
         <v>46316</v>
       </c>
+      <c r="U248" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="249" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A249" s="1">
@@ -14402,6 +15157,9 @@
       <c r="T249" s="1">
         <v>46316</v>
       </c>
+      <c r="U249" s="3" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="250" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A250" s="1">
@@ -14439,6 +15197,9 @@
       </c>
       <c r="R250" t="s">
         <v>38</v>
+      </c>
+      <c r="U250" s="3" t="s">
+        <v>696</v>
       </c>
       <c r="W250" t="s">
         <v>207</v>

</xml_diff>

<commit_message>
Kanban: folio DC-AB016 → 📨 Enviado a Cuentas por Pagar
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -5017,10 +5017,14 @@
       <c r="R65" t="inlineStr"/>
       <c r="S65" t="inlineStr"/>
       <c r="T65" t="inlineStr"/>
-      <c r="U65" t="inlineStr"/>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>28/09/2026 09:46</t>
+        </is>
+      </c>
       <c r="V65" t="inlineStr">
         <is>
-          <t>🗑️ En destrucción</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-MZ039: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -3218,7 +3218,11 @@
           <t>Recolección</t>
         </is>
       </c>
-      <c r="L40" t="inlineStr"/>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>8440</t>
+        </is>
+      </c>
       <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr"/>
       <c r="O40" t="inlineStr">
@@ -3239,7 +3243,7 @@
       <c r="T40" t="inlineStr"/>
       <c r="U40" t="inlineStr">
         <is>
-          <t>28/09/2026 09:46</t>
+          <t>28/09/2026 09:49</t>
         </is>
       </c>
       <c r="V40" t="inlineStr">

</xml_diff>

<commit_message>
Garantía DC-AB016: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -5002,7 +5002,11 @@
           <t>Recolección</t>
         </is>
       </c>
-      <c r="L65" t="inlineStr"/>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>8440</t>
+        </is>
+      </c>
       <c r="M65" t="inlineStr"/>
       <c r="N65" t="inlineStr"/>
       <c r="O65" t="inlineStr">
@@ -5023,7 +5027,7 @@
       <c r="T65" t="inlineStr"/>
       <c r="U65" t="inlineStr">
         <is>
-          <t>28/09/2026 09:46</t>
+          <t>28/09/2026 09:51</t>
         </is>
       </c>
       <c r="V65" t="inlineStr">

</xml_diff>

<commit_message>
Cuarentena: 4 folio(s) de GERARDO SOTO RAMOS liberados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1697,11 +1697,11 @@
         </is>
       </c>
       <c r="P18" s="1" t="n">
-        <v>46142</v>
+        <v>46293</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Cuarentena</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="R18" s="1" t="n">
@@ -1711,7 +1711,11 @@
         <v>46316</v>
       </c>
       <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr"/>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>28/09/2026 09:54</t>
+        </is>
+      </c>
       <c r="V18" t="inlineStr"/>
     </row>
     <row r="19">
@@ -9301,11 +9305,11 @@
         </is>
       </c>
       <c r="P126" s="1" t="n">
-        <v>46213</v>
+        <v>46293</v>
       </c>
       <c r="Q126" t="inlineStr">
         <is>
-          <t>Cuarentena</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="R126" s="1" t="n">
@@ -9315,7 +9319,11 @@
         <v>46316</v>
       </c>
       <c r="T126" t="inlineStr"/>
-      <c r="U126" t="inlineStr"/>
+      <c r="U126" t="inlineStr">
+        <is>
+          <t>28/09/2026 09:54</t>
+        </is>
+      </c>
       <c r="V126" t="inlineStr"/>
     </row>
     <row r="127">
@@ -12041,11 +12049,11 @@
       <c r="N168" t="inlineStr"/>
       <c r="O168" t="inlineStr"/>
       <c r="P168" s="1" t="n">
-        <v>46252</v>
+        <v>46293</v>
       </c>
       <c r="Q168" t="inlineStr">
         <is>
-          <t>Cuarentena</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="R168" s="1" t="n">
@@ -12055,7 +12063,11 @@
         <v>46316</v>
       </c>
       <c r="T168" t="inlineStr"/>
-      <c r="U168" t="inlineStr"/>
+      <c r="U168" t="inlineStr">
+        <is>
+          <t>28/09/2026 09:54</t>
+        </is>
+      </c>
       <c r="V168" t="inlineStr"/>
     </row>
     <row r="169">
@@ -14461,11 +14473,11 @@
       <c r="N208" t="inlineStr"/>
       <c r="O208" t="inlineStr"/>
       <c r="P208" s="1" t="n">
-        <v>46282</v>
+        <v>46293</v>
       </c>
       <c r="Q208" t="inlineStr">
         <is>
-          <t>Cuarentena</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="R208" s="1" t="n">
@@ -14475,7 +14487,11 @@
         <v>46316</v>
       </c>
       <c r="T208" t="inlineStr"/>
-      <c r="U208" t="inlineStr"/>
+      <c r="U208" t="inlineStr">
+        <is>
+          <t>28/09/2026 09:54</t>
+        </is>
+      </c>
       <c r="V208" t="inlineStr"/>
     </row>
     <row r="209">

</xml_diff>

<commit_message>
Cuarentena: 3 folio(s) regresados (DC-JN014, DC-JL020, DC-AG020)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1716,7 +1716,11 @@
           <t>28/09/2026 09:54</t>
         </is>
       </c>
-      <c r="V18" t="inlineStr"/>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>🚚 En recolección</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
@@ -9309,22 +9313,26 @@
       </c>
       <c r="Q126" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Cuarentena</t>
         </is>
       </c>
       <c r="R126" s="1" t="n">
-        <v>46286</v>
+        <v>46293</v>
       </c>
       <c r="S126" s="1" t="n">
-        <v>46316</v>
+        <v>46323</v>
       </c>
       <c r="T126" t="inlineStr"/>
       <c r="U126" t="inlineStr">
         <is>
-          <t>28/09/2026 09:54</t>
-        </is>
-      </c>
-      <c r="V126" t="inlineStr"/>
+          <t>28/09/2026 10:15</t>
+        </is>
+      </c>
+      <c r="V126" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="n">
@@ -12053,22 +12061,26 @@
       </c>
       <c r="Q168" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Cuarentena</t>
         </is>
       </c>
       <c r="R168" s="1" t="n">
-        <v>46286</v>
+        <v>46293</v>
       </c>
       <c r="S168" s="1" t="n">
-        <v>46316</v>
+        <v>46323</v>
       </c>
       <c r="T168" t="inlineStr"/>
       <c r="U168" t="inlineStr">
         <is>
-          <t>28/09/2026 09:54</t>
-        </is>
-      </c>
-      <c r="V168" t="inlineStr"/>
+          <t>28/09/2026 10:15</t>
+        </is>
+      </c>
+      <c r="V168" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="n">
@@ -14477,22 +14489,26 @@
       </c>
       <c r="Q208" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Cuarentena</t>
         </is>
       </c>
       <c r="R208" s="1" t="n">
-        <v>46286</v>
+        <v>46293</v>
       </c>
       <c r="S208" s="1" t="n">
-        <v>46316</v>
+        <v>46323</v>
       </c>
       <c r="T208" t="inlineStr"/>
       <c r="U208" t="inlineStr">
         <is>
-          <t>28/09/2026 09:54</t>
-        </is>
-      </c>
-      <c r="V208" t="inlineStr"/>
+          <t>28/09/2026 10:15</t>
+        </is>
+      </c>
+      <c r="V208" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="1" t="n">

</xml_diff>

<commit_message>
Garantía DC-MZ017: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1688,7 +1688,11 @@
           <t>Recolección</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr"/>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>8387</t>
+        </is>
+      </c>
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr">
@@ -1713,7 +1717,7 @@
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr">
         <is>
-          <t>28/09/2026 09:54</t>
+          <t>28/09/2026 11:36</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">

</xml_diff>

<commit_message>
Garantía DC-MZ030: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -2602,7 +2602,11 @@
           <t>Recolección</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>8397</t>
+        </is>
+      </c>
       <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr">
@@ -2621,7 +2625,11 @@
       <c r="R31" t="inlineStr"/>
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr"/>
-      <c r="U31" t="inlineStr"/>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>28/09/2026 11:45</t>
+        </is>
+      </c>
       <c r="V31" t="inlineStr">
         <is>
           <t>📨 Enviado a Cuentas por Pagar</t>

</xml_diff>

<commit_message>
Garantía DC-MY033: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -7836,7 +7836,11 @@
           <t>Recolección</t>
         </is>
       </c>
-      <c r="L105" t="inlineStr"/>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>8397</t>
+        </is>
+      </c>
       <c r="M105" t="inlineStr"/>
       <c r="N105" t="inlineStr"/>
       <c r="O105" t="inlineStr">
@@ -7855,7 +7859,11 @@
       <c r="R105" t="inlineStr"/>
       <c r="S105" t="inlineStr"/>
       <c r="T105" t="inlineStr"/>
-      <c r="U105" t="inlineStr"/>
+      <c r="U105" t="inlineStr">
+        <is>
+          <t>28/09/2026 11:45</t>
+        </is>
+      </c>
       <c r="V105" t="inlineStr">
         <is>
           <t>📨 Enviado a Cuentas por Pagar</t>

</xml_diff>

<commit_message>
Garantía DC-AB012: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -4740,7 +4740,11 @@
           <t>Recolección</t>
         </is>
       </c>
-      <c r="L61" t="inlineStr"/>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>8445</t>
+        </is>
+      </c>
       <c r="M61" t="inlineStr"/>
       <c r="N61" t="inlineStr"/>
       <c r="O61" t="inlineStr">
@@ -4759,10 +4763,14 @@
       <c r="R61" t="inlineStr"/>
       <c r="S61" t="inlineStr"/>
       <c r="T61" t="inlineStr"/>
-      <c r="U61" t="inlineStr"/>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>28/09/2026 11:47</t>
+        </is>
+      </c>
       <c r="V61" t="inlineStr">
         <is>
-          <t>🗑️ En destrucción</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-JN023: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -9832,7 +9832,11 @@
           <t>Recolección</t>
         </is>
       </c>
-      <c r="L133" t="inlineStr"/>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>8445</t>
+        </is>
+      </c>
       <c r="M133" t="inlineStr"/>
       <c r="N133" t="inlineStr"/>
       <c r="O133" t="inlineStr">
@@ -9851,7 +9855,11 @@
       <c r="R133" t="inlineStr"/>
       <c r="S133" t="inlineStr"/>
       <c r="T133" t="inlineStr"/>
-      <c r="U133" t="inlineStr"/>
+      <c r="U133" t="inlineStr">
+        <is>
+          <t>28/09/2026 11:48</t>
+        </is>
+      </c>
       <c r="V133" t="inlineStr">
         <is>
           <t>🗑️ En destrucción</t>

</xml_diff>

<commit_message>
Garantía DC-JL032: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -13676,7 +13676,11 @@
       </c>
       <c r="J194" t="inlineStr"/>
       <c r="K194" t="inlineStr"/>
-      <c r="L194" t="inlineStr"/>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>8445</t>
+        </is>
+      </c>
       <c r="M194" t="inlineStr"/>
       <c r="N194" t="inlineStr"/>
       <c r="O194" t="inlineStr"/>
@@ -13691,7 +13695,11 @@
       <c r="R194" t="inlineStr"/>
       <c r="S194" t="inlineStr"/>
       <c r="T194" t="inlineStr"/>
-      <c r="U194" t="inlineStr"/>
+      <c r="U194" t="inlineStr">
+        <is>
+          <t>28/09/2026 11:49</t>
+        </is>
+      </c>
       <c r="V194" t="inlineStr">
         <is>
           <t>📝 Reporte recibido</t>

</xml_diff>

<commit_message>
Garantía DC-AG029: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -16631,8 +16631,16 @@
         <v>46372</v>
       </c>
       <c r="J243" t="inlineStr"/>
-      <c r="K243" t="inlineStr"/>
-      <c r="L243" t="inlineStr"/>
+      <c r="K243" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L243" t="inlineStr">
+        <is>
+          <t>8445</t>
+        </is>
+      </c>
       <c r="M243" t="inlineStr"/>
       <c r="N243" t="inlineStr"/>
       <c r="O243" t="inlineStr"/>
@@ -16647,10 +16655,14 @@
       <c r="R243" t="inlineStr"/>
       <c r="S243" t="inlineStr"/>
       <c r="T243" t="inlineStr"/>
-      <c r="U243" t="inlineStr"/>
+      <c r="U243" t="inlineStr">
+        <is>
+          <t>28/09/2026 11:50</t>
+        </is>
+      </c>
       <c r="V243" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-JN018: Folio marcado como RESUELTO (fecha cierre 28/09/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -9622,7 +9622,11 @@
         </is>
       </c>
       <c r="M130" t="inlineStr"/>
-      <c r="N130" t="inlineStr"/>
+      <c r="N130" t="inlineStr">
+        <is>
+          <t>223118</t>
+        </is>
+      </c>
       <c r="O130" t="inlineStr">
         <is>
           <t>DEVOLUCION 8374</t>
@@ -9633,13 +9637,19 @@
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R130" t="inlineStr"/>
       <c r="S130" t="inlineStr"/>
-      <c r="T130" t="inlineStr"/>
-      <c r="U130" t="inlineStr"/>
+      <c r="T130" s="1" t="n">
+        <v>46293</v>
+      </c>
+      <c r="U130" t="inlineStr">
+        <is>
+          <t>28/09/2026 12:34</t>
+        </is>
+      </c>
       <c r="V130" t="inlineStr">
         <is>
           <t>📨 Enviado a Cuentas por Pagar</t>

</xml_diff>

<commit_message>
Garantía DC-MZ002: Folio marcado como RESUELTO (fecha cierre 28/09/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -656,7 +656,11 @@
         </is>
       </c>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>5f751644</t>
+        </is>
+      </c>
       <c r="O3" t="inlineStr">
         <is>
           <t>DEVOLUCION  8325 | [21/07/2026 11:16 · Reactivación] Etapa 'Destino final' reactivada | [17/08/2026 17:33 · Fernando] Avance en Cuentas por pagar | [17/08/2026 17:57 · Yolanda] Avance en Cuentas por pagar</t>
@@ -667,13 +671,19 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
+      <c r="T3" s="1" t="n">
+        <v>46293</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>28/09/2026 12:36</t>
+        </is>
+      </c>
       <c r="V3" t="inlineStr">
         <is>
           <t>📨 Enviado a Cuentas por Pagar</t>

</xml_diff>

<commit_message>
Garantía DC-AB007: Folio marcado como RESUELTO (fecha cierre 28/09/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -4396,7 +4396,11 @@
         </is>
       </c>
       <c r="M56" t="inlineStr"/>
-      <c r="N56" t="inlineStr"/>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>5f751644</t>
+        </is>
+      </c>
       <c r="O56" t="inlineStr">
         <is>
           <t>DEVOLUCION  8325</t>
@@ -4407,13 +4411,19 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R56" t="inlineStr"/>
       <c r="S56" t="inlineStr"/>
-      <c r="T56" t="inlineStr"/>
-      <c r="U56" t="inlineStr"/>
+      <c r="T56" s="1" t="n">
+        <v>46293</v>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>28/09/2026 12:36</t>
+        </is>
+      </c>
       <c r="V56" t="inlineStr">
         <is>
           <t>📨 Enviado a Cuentas por Pagar</t>

</xml_diff>

<commit_message>
Garantía DC-AG030: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -16602,7 +16602,11 @@
       </c>
       <c r="J242" t="inlineStr"/>
       <c r="K242" t="inlineStr"/>
-      <c r="L242" t="inlineStr"/>
+      <c r="L242" t="inlineStr">
+        <is>
+          <t>8410</t>
+        </is>
+      </c>
       <c r="M242" t="inlineStr"/>
       <c r="N242" t="inlineStr"/>
       <c r="O242" t="inlineStr"/>
@@ -16617,10 +16621,14 @@
       <c r="R242" t="inlineStr"/>
       <c r="S242" t="inlineStr"/>
       <c r="T242" t="inlineStr"/>
-      <c r="U242" t="inlineStr"/>
+      <c r="U242" t="inlineStr">
+        <is>
+          <t>28/09/2026 12:49</t>
+        </is>
+      </c>
       <c r="V242" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cuarentena: 1 folio(s) de INTERRUPTORES Y GABINETES ELECTRICOS SA DE CV liberados (DC-AB038)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -6413,11 +6413,11 @@
         </is>
       </c>
       <c r="P84" s="1" t="n">
-        <v>46162</v>
+        <v>46293</v>
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t>Cuarentena</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="R84" s="1" t="n">
@@ -6427,7 +6427,11 @@
         <v>46316</v>
       </c>
       <c r="T84" t="inlineStr"/>
-      <c r="U84" t="inlineStr"/>
+      <c r="U84" t="inlineStr">
+        <is>
+          <t>28/09/2026 12:49</t>
+        </is>
+      </c>
       <c r="V84" t="inlineStr"/>
     </row>
     <row r="85">

</xml_diff>

<commit_message>
Garantía DC-AB038: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -6429,10 +6429,14 @@
       <c r="T84" t="inlineStr"/>
       <c r="U84" t="inlineStr">
         <is>
-          <t>28/09/2026 12:49</t>
-        </is>
-      </c>
-      <c r="V84" t="inlineStr"/>
+          <t>28/09/2026 13:01</t>
+        </is>
+      </c>
+      <c r="V84" t="inlineStr">
+        <is>
+          <t>📨 Enviado a Cuentas por Pagar</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="n">

</xml_diff>

<commit_message>
Cuarentena: 1 folio(s) de MARIBEL CONTRERAS SOTO liberados (DC-AG034)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -16435,11 +16435,11 @@
       <c r="N239" t="inlineStr"/>
       <c r="O239" t="inlineStr"/>
       <c r="P239" s="1" t="n">
-        <v>46282</v>
+        <v>46293</v>
       </c>
       <c r="Q239" t="inlineStr">
         <is>
-          <t>Cuarentena</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="R239" s="1" t="n">
@@ -16449,7 +16449,11 @@
         <v>46316</v>
       </c>
       <c r="T239" t="inlineStr"/>
-      <c r="U239" t="inlineStr"/>
+      <c r="U239" t="inlineStr">
+        <is>
+          <t>28/09/2026 13:05</t>
+        </is>
+      </c>
       <c r="V239" t="inlineStr"/>
     </row>
     <row r="240">

</xml_diff>

<commit_message>
Garantía DC-AG034: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -16429,8 +16429,16 @@
         <v>46372</v>
       </c>
       <c r="J239" t="inlineStr"/>
-      <c r="K239" t="inlineStr"/>
-      <c r="L239" t="inlineStr"/>
+      <c r="K239" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L239" t="inlineStr">
+        <is>
+          <t>8440</t>
+        </is>
+      </c>
       <c r="M239" t="inlineStr"/>
       <c r="N239" t="inlineStr"/>
       <c r="O239" t="inlineStr"/>
@@ -16451,10 +16459,14 @@
       <c r="T239" t="inlineStr"/>
       <c r="U239" t="inlineStr">
         <is>
-          <t>28/09/2026 13:05</t>
-        </is>
-      </c>
-      <c r="V239" t="inlineStr"/>
+          <t>28/09/2026 13:08</t>
+        </is>
+      </c>
+      <c r="V239" t="inlineStr">
+        <is>
+          <t>📨 Enviado a Cuentas por Pagar</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="1" t="n">

</xml_diff>

<commit_message>
Garantía DC-JL048: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -12253,8 +12253,16 @@
         <v>46342</v>
       </c>
       <c r="J170" t="inlineStr"/>
-      <c r="K170" t="inlineStr"/>
-      <c r="L170" t="inlineStr"/>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>8433</t>
+        </is>
+      </c>
       <c r="M170" t="inlineStr"/>
       <c r="N170" t="inlineStr"/>
       <c r="O170" t="inlineStr"/>
@@ -12269,10 +12277,14 @@
       <c r="R170" t="inlineStr"/>
       <c r="S170" t="inlineStr"/>
       <c r="T170" t="inlineStr"/>
-      <c r="U170" t="inlineStr"/>
+      <c r="U170" t="inlineStr">
+        <is>
+          <t>28/09/2026 13:10</t>
+        </is>
+      </c>
       <c r="V170" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cuarentena: 2 folio(s) de CNX INTERNACIONAL SA DE CV liberados (DC-AB022, DC-MY011)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -5507,11 +5507,11 @@
         </is>
       </c>
       <c r="P71" s="1" t="n">
-        <v>46162</v>
+        <v>46293</v>
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>Cuarentena</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="R71" s="1" t="n">
@@ -5521,7 +5521,11 @@
         <v>46316</v>
       </c>
       <c r="T71" t="inlineStr"/>
-      <c r="U71" t="inlineStr"/>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>28/09/2026 13:14</t>
+        </is>
+      </c>
       <c r="V71" t="inlineStr"/>
     </row>
     <row r="72">
@@ -7111,11 +7115,11 @@
         </is>
       </c>
       <c r="P94" s="1" t="n">
-        <v>46195</v>
+        <v>46293</v>
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t>Cuarentena</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="R94" s="1" t="n">
@@ -7125,7 +7129,11 @@
         <v>46316</v>
       </c>
       <c r="T94" t="inlineStr"/>
-      <c r="U94" t="inlineStr"/>
+      <c r="U94" t="inlineStr">
+        <is>
+          <t>28/09/2026 13:14</t>
+        </is>
+      </c>
       <c r="V94" t="inlineStr"/>
     </row>
     <row r="95">

</xml_diff>

<commit_message>
Garantía DC-AB022: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -5523,10 +5523,14 @@
       <c r="T71" t="inlineStr"/>
       <c r="U71" t="inlineStr">
         <is>
-          <t>28/09/2026 13:14</t>
-        </is>
-      </c>
-      <c r="V71" t="inlineStr"/>
+          <t>28/09/2026 13:16</t>
+        </is>
+      </c>
+      <c r="V71" t="inlineStr">
+        <is>
+          <t>📨 Enviado a Cuentas por Pagar</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
@@ -7134,7 +7138,11 @@
           <t>28/09/2026 13:14</t>
         </is>
       </c>
-      <c r="V94" t="inlineStr"/>
+      <c r="V94" t="inlineStr">
+        <is>
+          <t>🚚 En recolección</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="n">

</xml_diff>

<commit_message>
Garantía DC-MY011: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -7110,7 +7110,11 @@
           <t>Recolección</t>
         </is>
       </c>
-      <c r="L94" t="inlineStr"/>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>8427</t>
+        </is>
+      </c>
       <c r="M94" t="inlineStr"/>
       <c r="N94" t="inlineStr"/>
       <c r="O94" t="inlineStr">
@@ -7135,12 +7139,12 @@
       <c r="T94" t="inlineStr"/>
       <c r="U94" t="inlineStr">
         <is>
-          <t>28/09/2026 13:14</t>
+          <t>28/09/2026 13:16</t>
         </is>
       </c>
       <c r="V94" t="inlineStr">
         <is>
-          <t>🚚 En recolección</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-JN006: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -9024,7 +9024,11 @@
           <t>Recolección</t>
         </is>
       </c>
-      <c r="L121" t="inlineStr"/>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>8427</t>
+        </is>
+      </c>
       <c r="M121" t="inlineStr"/>
       <c r="N121" t="inlineStr"/>
       <c r="O121" t="inlineStr">
@@ -9043,7 +9047,11 @@
       <c r="R121" t="inlineStr"/>
       <c r="S121" t="inlineStr"/>
       <c r="T121" t="inlineStr"/>
-      <c r="U121" t="inlineStr"/>
+      <c r="U121" t="inlineStr">
+        <is>
+          <t>28/09/2026 13:17</t>
+        </is>
+      </c>
       <c r="V121" t="inlineStr">
         <is>
           <t>📨 Enviado a Cuentas por Pagar</t>

</xml_diff>

<commit_message>
Garantía DC-MY016: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -7262,7 +7262,11 @@
           <t>Recolección</t>
         </is>
       </c>
-      <c r="L96" t="inlineStr"/>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>8844</t>
+        </is>
+      </c>
       <c r="M96" t="inlineStr"/>
       <c r="N96" t="inlineStr"/>
       <c r="O96" t="inlineStr">
@@ -7281,10 +7285,14 @@
       <c r="R96" t="inlineStr"/>
       <c r="S96" t="inlineStr"/>
       <c r="T96" t="inlineStr"/>
-      <c r="U96" t="inlineStr"/>
+      <c r="U96" t="inlineStr">
+        <is>
+          <t>28/09/2026 14:56</t>
+        </is>
+      </c>
       <c r="V96" t="inlineStr">
         <is>
-          <t>🗑️ En destrucción</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-JL017: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -11673,11 +11673,19 @@
         <v>46342</v>
       </c>
       <c r="J160" t="inlineStr"/>
-      <c r="K160" t="inlineStr"/>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>Destrucción</t>
+        </is>
+      </c>
       <c r="L160" t="inlineStr"/>
       <c r="M160" t="inlineStr"/>
       <c r="N160" t="inlineStr"/>
-      <c r="O160" t="inlineStr"/>
+      <c r="O160" t="inlineStr">
+        <is>
+          <t>Descontar en proximo pago se envio correo 30/09 facturas para pago en Octubre</t>
+        </is>
+      </c>
       <c r="P160" s="1" t="n">
         <v>46252</v>
       </c>
@@ -11689,10 +11697,14 @@
       <c r="R160" t="inlineStr"/>
       <c r="S160" t="inlineStr"/>
       <c r="T160" t="inlineStr"/>
-      <c r="U160" t="inlineStr"/>
+      <c r="U160" t="inlineStr">
+        <is>
+          <t>30/09/2026 11:24</t>
+        </is>
+      </c>
       <c r="V160" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-AB025: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -5714,7 +5714,11 @@
           <t>Destrucción</t>
         </is>
       </c>
-      <c r="L74" t="inlineStr"/>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>8307</t>
+        </is>
+      </c>
       <c r="M74" t="inlineStr"/>
       <c r="N74" t="inlineStr"/>
       <c r="O74" t="inlineStr">
@@ -5733,10 +5737,14 @@
       <c r="R74" t="inlineStr"/>
       <c r="S74" t="inlineStr"/>
       <c r="T74" t="inlineStr"/>
-      <c r="U74" t="inlineStr"/>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>30/09/2026 11:40</t>
+        </is>
+      </c>
       <c r="V74" t="inlineStr">
         <is>
-          <t>🗑️ En destrucción</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-JL029: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -11383,9 +11383,17 @@
       <c r="J155" t="inlineStr"/>
       <c r="K155" t="inlineStr"/>
       <c r="L155" t="inlineStr"/>
-      <c r="M155" t="inlineStr"/>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>37554</t>
+        </is>
+      </c>
       <c r="N155" t="inlineStr"/>
-      <c r="O155" t="inlineStr"/>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>TREASPASO ALMACEN  37554  AGOSTO  HIZO CAMBIO FISICO</t>
+        </is>
+      </c>
       <c r="P155" s="1" t="n">
         <v>46252</v>
       </c>
@@ -11397,10 +11405,14 @@
       <c r="R155" t="inlineStr"/>
       <c r="S155" t="inlineStr"/>
       <c r="T155" t="inlineStr"/>
-      <c r="U155" t="inlineStr"/>
+      <c r="U155" t="inlineStr">
+        <is>
+          <t>02/10/2026 11:17</t>
+        </is>
+      </c>
       <c r="V155" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-JL029: Folio marcado como RESUELTO (con NC, fecha cierre 27/08/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -11388,7 +11388,11 @@
           <t>37554</t>
         </is>
       </c>
-      <c r="N155" t="inlineStr"/>
+      <c r="N155" t="inlineStr">
+        <is>
+          <t>37554</t>
+        </is>
+      </c>
       <c r="O155" t="inlineStr">
         <is>
           <t>TREASPASO ALMACEN  37554  AGOSTO  HIZO CAMBIO FISICO</t>
@@ -11399,15 +11403,17 @@
       </c>
       <c r="Q155" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R155" t="inlineStr"/>
       <c r="S155" t="inlineStr"/>
-      <c r="T155" t="inlineStr"/>
+      <c r="T155" s="1" t="n">
+        <v>46261</v>
+      </c>
       <c r="U155" t="inlineStr">
         <is>
-          <t>02/10/2026 11:17</t>
+          <t>02/10/2026 11:18</t>
         </is>
       </c>
       <c r="V155" t="inlineStr">

</xml_diff>

<commit_message>
Garantía DC-AG027: Folio marcado como RESUELTO (fecha cierre 02/10/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -16854,20 +16854,30 @@
       <c r="K244" t="inlineStr"/>
       <c r="L244" t="inlineStr"/>
       <c r="M244" t="inlineStr"/>
-      <c r="N244" t="inlineStr"/>
+      <c r="N244" t="inlineStr">
+        <is>
+          <t>38204</t>
+        </is>
+      </c>
       <c r="O244" t="inlineStr"/>
       <c r="P244" s="1" t="n">
         <v>46282</v>
       </c>
       <c r="Q244" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R244" t="inlineStr"/>
       <c r="S244" t="inlineStr"/>
-      <c r="T244" t="inlineStr"/>
-      <c r="U244" t="inlineStr"/>
+      <c r="T244" s="1" t="n">
+        <v>46297</v>
+      </c>
+      <c r="U244" t="inlineStr">
+        <is>
+          <t>02/10/2026 11:21</t>
+        </is>
+      </c>
       <c r="V244" t="inlineStr">
         <is>
           <t>📝 Reporte recibido</t>

</xml_diff>

<commit_message>
Garantía DC-MZ027: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -2429,8 +2429,16 @@
       <c r="T28" s="1" t="n">
         <v>46199</v>
       </c>
-      <c r="U28" t="inlineStr"/>
-      <c r="V28" t="inlineStr"/>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>02/10/2026 11:21</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">

</xml_diff>

<commit_message>
Garantía DC-MZ040: Folio marcado como RESUELTO (fecha cierre 22/09/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -3340,7 +3340,11 @@
         </is>
       </c>
       <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>48936</t>
+        </is>
+      </c>
       <c r="O41" t="inlineStr">
         <is>
           <t>DEVOLUCION 8367</t>
@@ -3351,13 +3355,19 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R41" t="inlineStr"/>
       <c r="S41" t="inlineStr"/>
-      <c r="T41" t="inlineStr"/>
-      <c r="U41" t="inlineStr"/>
+      <c r="T41" s="1" t="n">
+        <v>46287</v>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>02/10/2026 11:32</t>
+        </is>
+      </c>
       <c r="V41" t="inlineStr">
         <is>
           <t>📨 Enviado a Cuentas por Pagar</t>

</xml_diff>

<commit_message>
Garantía DC-AB017: Folio marcado como RESUELTO (fecha cierre 22/09/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -5152,7 +5152,11 @@
         </is>
       </c>
       <c r="M66" t="inlineStr"/>
-      <c r="N66" t="inlineStr"/>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>48936</t>
+        </is>
+      </c>
       <c r="O66" t="inlineStr">
         <is>
           <t>DEVOLUCION 8367</t>
@@ -5163,13 +5167,19 @@
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R66" t="inlineStr"/>
       <c r="S66" t="inlineStr"/>
-      <c r="T66" t="inlineStr"/>
-      <c r="U66" t="inlineStr"/>
+      <c r="T66" s="1" t="n">
+        <v>46287</v>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>02/10/2026 11:33</t>
+        </is>
+      </c>
       <c r="V66" t="inlineStr">
         <is>
           <t>📨 Enviado a Cuentas por Pagar</t>

</xml_diff>

<commit_message>
Casos especiales: + MARIBEL CONTRERAS SOTO (Descuento en siguiente compra)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -10,6 +10,7 @@
     <sheet name="datos- FOLIO DE GARANTIA" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="FOLIOS DE DEVOLUCION-GARANTIA" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="NC PENDIENTES" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="CASOS ESPECIALES" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30900,4 +30901,60 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>PROVEEDOR</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>TIPO</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>MOTIVO</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>FECHA MARCADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MARIBEL CONTRERAS SOTO</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Descuento en siguiente compra</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Se descuentan las devoluciones en las siguientes compras y se le compra cada 6 meses</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>46297</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Garantía DC-JL023: Folio marcado como RESUELTO (con NC, fecha cierre 03/10/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -12548,26 +12548,44 @@
         <v>46342</v>
       </c>
       <c r="J173" t="inlineStr"/>
-      <c r="K173" t="inlineStr"/>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>Destrucción</t>
+        </is>
+      </c>
       <c r="L173" t="inlineStr"/>
       <c r="M173" t="inlineStr"/>
-      <c r="N173" t="inlineStr"/>
-      <c r="O173" t="inlineStr"/>
+      <c r="N173" t="inlineStr">
+        <is>
+          <t>37771- 37772</t>
+        </is>
+      </c>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>destruccion nc-37771-37772</t>
+        </is>
+      </c>
       <c r="P173" s="1" t="n">
         <v>46252</v>
       </c>
       <c r="Q173" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R173" t="inlineStr"/>
       <c r="S173" t="inlineStr"/>
-      <c r="T173" t="inlineStr"/>
-      <c r="U173" t="inlineStr"/>
+      <c r="T173" s="1" t="n">
+        <v>46298</v>
+      </c>
+      <c r="U173" t="inlineStr">
+        <is>
+          <t>03/10/2026 11:48</t>
+        </is>
+      </c>
       <c r="V173" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-JL023: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -12555,11 +12555,7 @@
       </c>
       <c r="L173" t="inlineStr"/>
       <c r="M173" t="inlineStr"/>
-      <c r="N173" t="inlineStr">
-        <is>
-          <t>37771- 37772</t>
-        </is>
-      </c>
+      <c r="N173" t="inlineStr"/>
       <c r="O173" t="inlineStr">
         <is>
           <t>destruccion nc-37771-37772</t>
@@ -12580,7 +12576,7 @@
       </c>
       <c r="U173" t="inlineStr">
         <is>
-          <t>03/10/2026 11:48</t>
+          <t>03/10/2026 11:49</t>
         </is>
       </c>
       <c r="V173" t="inlineStr">

</xml_diff>

<commit_message>
Garantía DC-AG024: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -15958,11 +15958,19 @@
         <v>46372</v>
       </c>
       <c r="J229" t="inlineStr"/>
-      <c r="K229" t="inlineStr"/>
+      <c r="K229" t="inlineStr">
+        <is>
+          <t>Destrucción</t>
+        </is>
+      </c>
       <c r="L229" t="inlineStr"/>
       <c r="M229" t="inlineStr"/>
       <c r="N229" t="inlineStr"/>
-      <c r="O229" t="inlineStr"/>
+      <c r="O229" t="inlineStr">
+        <is>
+          <t>destruccion  NC- 37771</t>
+        </is>
+      </c>
       <c r="P229" s="1" t="n">
         <v>46282</v>
       </c>
@@ -15974,10 +15982,14 @@
       <c r="R229" t="inlineStr"/>
       <c r="S229" t="inlineStr"/>
       <c r="T229" t="inlineStr"/>
-      <c r="U229" t="inlineStr"/>
+      <c r="U229" t="inlineStr">
+        <is>
+          <t>03/10/2026 12:08</t>
+        </is>
+      </c>
       <c r="V229" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-JL038: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -10924,7 +10924,7 @@
       <c r="N147" t="inlineStr"/>
       <c r="O147" t="inlineStr">
         <is>
-          <t>[25/08/2026 08:53 · Francisco] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [29/08/2026 13:02 · Francisco] Etapa 2 TERMINADA · Destrucción → pasa a Disposición final</t>
+          <t>nc -DM30496035</t>
         </is>
       </c>
       <c r="P147" s="1" t="n">
@@ -10938,10 +10938,14 @@
       <c r="R147" t="inlineStr"/>
       <c r="S147" t="inlineStr"/>
       <c r="T147" t="inlineStr"/>
-      <c r="U147" t="inlineStr"/>
+      <c r="U147" t="inlineStr">
+        <is>
+          <t>03/10/2026 12:19</t>
+        </is>
+      </c>
       <c r="V147" t="inlineStr">
         <is>
-          <t>🗑️ En destrucción</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>
@@ -12558,7 +12562,7 @@
       <c r="N173" t="inlineStr"/>
       <c r="O173" t="inlineStr">
         <is>
-          <t>destrucción nc-37771-37772</t>
+          <t>destruccion nc-37771-37772</t>
         </is>
       </c>
       <c r="P173" s="1" t="n">
@@ -12576,7 +12580,7 @@
       </c>
       <c r="U173" t="inlineStr">
         <is>
-          <t>03/10/2026 12:19</t>
+          <t>03/10/2026 11:52</t>
         </is>
       </c>
       <c r="V173" t="inlineStr">

</xml_diff>

<commit_message>
Cuarentena: 1 folio(s) de KWIKSET RESIDENCIAL MEXICO SA DE CV liberados (DC-JN028)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -10170,11 +10170,11 @@
         </is>
       </c>
       <c r="P136" s="1" t="n">
-        <v>46213</v>
+        <v>46298</v>
       </c>
       <c r="Q136" t="inlineStr">
         <is>
-          <t>Cuarentena</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="R136" s="1" t="n">
@@ -10184,7 +10184,11 @@
         <v>46316</v>
       </c>
       <c r="T136" t="inlineStr"/>
-      <c r="U136" t="inlineStr"/>
+      <c r="U136" t="inlineStr">
+        <is>
+          <t>03/10/2026 12:20</t>
+        </is>
+      </c>
       <c r="V136" t="inlineStr"/>
     </row>
     <row r="137">

</xml_diff>

<commit_message>
Garantía DC-JN028: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -10158,7 +10158,7 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>Recolección</t>
+          <t>Destrucción</t>
         </is>
       </c>
       <c r="L136" t="inlineStr"/>
@@ -10166,7 +10166,7 @@
       <c r="N136" t="inlineStr"/>
       <c r="O136" t="inlineStr">
         <is>
-          <t>DEVOLUCION</t>
+          <t>DESTRUCCION  RM-30496035</t>
         </is>
       </c>
       <c r="P136" s="1" t="n">
@@ -10186,10 +10186,14 @@
       <c r="T136" t="inlineStr"/>
       <c r="U136" t="inlineStr">
         <is>
-          <t>03/10/2026 12:20</t>
-        </is>
-      </c>
-      <c r="V136" t="inlineStr"/>
+          <t>03/10/2026 12:22</t>
+        </is>
+      </c>
+      <c r="V136" t="inlineStr">
+        <is>
+          <t>📨 Enviado a Cuentas por Pagar</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="n">

</xml_diff>

<commit_message>
Garantía DC-JL023: Folio reabierto desde Resuelto → 📨 Enviado a Cuentas por Pagar
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -12578,17 +12578,15 @@
       </c>
       <c r="Q173" t="inlineStr">
         <is>
-          <t>Resuelto</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="R173" t="inlineStr"/>
       <c r="S173" t="inlineStr"/>
-      <c r="T173" s="1" t="n">
-        <v>46298</v>
-      </c>
+      <c r="T173" t="inlineStr"/>
       <c r="U173" t="inlineStr">
         <is>
-          <t>03/10/2026 11:52</t>
+          <t>03/10/2026 12:27</t>
         </is>
       </c>
       <c r="V173" t="inlineStr">

</xml_diff>

<commit_message>
Garantía DC-JN002: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -8797,12 +8797,16 @@
           <t>Recolección</t>
         </is>
       </c>
-      <c r="L117" t="inlineStr"/>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>8451</t>
+        </is>
+      </c>
       <c r="M117" t="inlineStr"/>
       <c r="N117" t="inlineStr"/>
       <c r="O117" t="inlineStr">
         <is>
-          <t>DEVOLUCION</t>
+          <t>8451  DEVOLUCION</t>
         </is>
       </c>
       <c r="P117" s="1" t="n">
@@ -8816,10 +8820,14 @@
       <c r="R117" t="inlineStr"/>
       <c r="S117" t="inlineStr"/>
       <c r="T117" t="inlineStr"/>
-      <c r="U117" t="inlineStr"/>
+      <c r="U117" t="inlineStr">
+        <is>
+          <t>04/10/2026 22:34</t>
+        </is>
+      </c>
       <c r="V117" t="inlineStr">
         <is>
-          <t>🗑️ En destrucción</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-JL003: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -11007,12 +11007,16 @@
           <t>Recolección</t>
         </is>
       </c>
-      <c r="L148" t="inlineStr"/>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>8451</t>
+        </is>
+      </c>
       <c r="M148" t="inlineStr"/>
       <c r="N148" t="inlineStr"/>
       <c r="O148" t="inlineStr">
         <is>
-          <t>[25/08/2026 08:54 · Francisco] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [29/08/2026 13:03 · Francisco] Avance en Gestión</t>
+          <t>8451 Devolucion</t>
         </is>
       </c>
       <c r="P148" s="1" t="n">
@@ -11026,10 +11030,14 @@
       <c r="R148" t="inlineStr"/>
       <c r="S148" t="inlineStr"/>
       <c r="T148" t="inlineStr"/>
-      <c r="U148" t="inlineStr"/>
+      <c r="U148" t="inlineStr">
+        <is>
+          <t>04/10/2026 22:36</t>
+        </is>
+      </c>
       <c r="V148" t="inlineStr">
         <is>
-          <t>⏳ Esperando respuesta</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-AG002: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -15204,11 +15204,23 @@
         <v>46372</v>
       </c>
       <c r="J216" t="inlineStr"/>
-      <c r="K216" t="inlineStr"/>
-      <c r="L216" t="inlineStr"/>
+      <c r="K216" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L216" t="inlineStr">
+        <is>
+          <t>8451</t>
+        </is>
+      </c>
       <c r="M216" t="inlineStr"/>
       <c r="N216" t="inlineStr"/>
-      <c r="O216" t="inlineStr"/>
+      <c r="O216" t="inlineStr">
+        <is>
+          <t>8451 Devolucion</t>
+        </is>
+      </c>
       <c r="P216" s="1" t="n">
         <v>46282</v>
       </c>
@@ -15220,10 +15232,14 @@
       <c r="R216" t="inlineStr"/>
       <c r="S216" t="inlineStr"/>
       <c r="T216" t="inlineStr"/>
-      <c r="U216" t="inlineStr"/>
+      <c r="U216" t="inlineStr">
+        <is>
+          <t>04/10/2026 22:38</t>
+        </is>
+      </c>
       <c r="V216" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-JL015: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -11258,11 +11258,23 @@
         <v>46342</v>
       </c>
       <c r="J152" t="inlineStr"/>
-      <c r="K152" t="inlineStr"/>
-      <c r="L152" t="inlineStr"/>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>8453</t>
+        </is>
+      </c>
       <c r="M152" t="inlineStr"/>
       <c r="N152" t="inlineStr"/>
-      <c r="O152" t="inlineStr"/>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>8453 Devolucion</t>
+        </is>
+      </c>
       <c r="P152" s="1" t="n">
         <v>46252</v>
       </c>
@@ -11274,10 +11286,14 @@
       <c r="R152" t="inlineStr"/>
       <c r="S152" t="inlineStr"/>
       <c r="T152" t="inlineStr"/>
-      <c r="U152" t="inlineStr"/>
+      <c r="U152" t="inlineStr">
+        <is>
+          <t>04/10/2026 23:26</t>
+        </is>
+      </c>
       <c r="V152" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-AG017: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -16148,11 +16148,23 @@
         <v>46372</v>
       </c>
       <c r="J231" t="inlineStr"/>
-      <c r="K231" t="inlineStr"/>
-      <c r="L231" t="inlineStr"/>
+      <c r="K231" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L231" t="inlineStr">
+        <is>
+          <t>8453 -8454</t>
+        </is>
+      </c>
       <c r="M231" t="inlineStr"/>
       <c r="N231" t="inlineStr"/>
-      <c r="O231" t="inlineStr"/>
+      <c r="O231" t="inlineStr">
+        <is>
+          <t>8453-8454 Devolucion</t>
+        </is>
+      </c>
       <c r="P231" s="1" t="n">
         <v>46282</v>
       </c>
@@ -16164,10 +16176,14 @@
       <c r="R231" t="inlineStr"/>
       <c r="S231" t="inlineStr"/>
       <c r="T231" t="inlineStr"/>
-      <c r="U231" t="inlineStr"/>
+      <c r="U231" t="inlineStr">
+        <is>
+          <t>04/10/2026 23:29</t>
+        </is>
+      </c>
       <c r="V231" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cuarentena: 1 folio(s) de INDUSTRIAL DE TERMINALES, S.A. DE C.V. liberados (DC-JL024)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -13038,11 +13038,11 @@
         </is>
       </c>
       <c r="P180" s="1" t="n">
-        <v>46252</v>
+        <v>46299</v>
       </c>
       <c r="Q180" t="inlineStr">
         <is>
-          <t>Cuarentena</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="R180" s="1" t="n">
@@ -13052,7 +13052,11 @@
         <v>46316</v>
       </c>
       <c r="T180" t="inlineStr"/>
-      <c r="U180" t="inlineStr"/>
+      <c r="U180" t="inlineStr">
+        <is>
+          <t>04/10/2026 23:46</t>
+        </is>
+      </c>
       <c r="V180" t="inlineStr"/>
     </row>
     <row r="181">

</xml_diff>

<commit_message>
Garantía DC-JL024: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -13029,12 +13029,16 @@
           <t>Recolección</t>
         </is>
       </c>
-      <c r="L180" t="inlineStr"/>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>8411</t>
+        </is>
+      </c>
       <c r="M180" t="inlineStr"/>
       <c r="N180" t="inlineStr"/>
       <c r="O180" t="inlineStr">
         <is>
-          <t>[01/09/2026 10:16 · Admin cuarentena] Duración de cuarentena de INDUSTRIAL DE TERMINALES, S.A. DE C.V. ajustada a 29 días | [01/09/2026 10:16 · Admin cuarentena] 1 reclamación(es) de INDUSTRIAL DE TERMINALES, S.A. DE C.V. liberadas de cuarentena → Reporte de reclamo | [01/09/2026 10:18 · yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/09/2026 10:18 · yolanda] Etapa 2 TERMINADA · Recolección → pasa a Disposición final | [01/09/2026 10:19 · yolanda] Etapa Disposición final TERMINADA → pasa a Cuentas por pagar</t>
+          <t>8411 Devolucion</t>
         </is>
       </c>
       <c r="P180" s="1" t="n">
@@ -13054,10 +13058,14 @@
       <c r="T180" t="inlineStr"/>
       <c r="U180" t="inlineStr">
         <is>
-          <t>04/10/2026 23:46</t>
-        </is>
-      </c>
-      <c r="V180" t="inlineStr"/>
+          <t>04/10/2026 23:49</t>
+        </is>
+      </c>
+      <c r="V180" t="inlineStr">
+        <is>
+          <t>📨 Enviado a Cuentas por Pagar</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="1" t="n">

</xml_diff>

<commit_message>
Garantía DC-JL025: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -11138,7 +11138,11 @@
         <v>46342</v>
       </c>
       <c r="J150" t="inlineStr"/>
-      <c r="K150" t="inlineStr"/>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="L150" t="inlineStr"/>
       <c r="M150" t="inlineStr"/>
       <c r="N150" t="inlineStr"/>
@@ -11154,10 +11158,14 @@
       <c r="R150" t="inlineStr"/>
       <c r="S150" t="inlineStr"/>
       <c r="T150" t="inlineStr"/>
-      <c r="U150" t="inlineStr"/>
+      <c r="U150" t="inlineStr">
+        <is>
+          <t>04/10/2026 23:53</t>
+        </is>
+      </c>
       <c r="V150" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>🚚 En recolección</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-JL026: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -13112,15 +13112,15 @@
         <v>46342</v>
       </c>
       <c r="J181" t="inlineStr"/>
-      <c r="K181" t="inlineStr"/>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>Destrucción</t>
+        </is>
+      </c>
       <c r="L181" t="inlineStr"/>
       <c r="M181" t="inlineStr"/>
       <c r="N181" t="inlineStr"/>
-      <c r="O181" t="inlineStr">
-        <is>
-          <t>[25/08/2026 08:56 · Francisco] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
-        </is>
-      </c>
+      <c r="O181" t="inlineStr"/>
       <c r="P181" s="1" t="n">
         <v>46252</v>
       </c>
@@ -13132,10 +13132,14 @@
       <c r="R181" t="inlineStr"/>
       <c r="S181" t="inlineStr"/>
       <c r="T181" t="inlineStr"/>
-      <c r="U181" t="inlineStr"/>
+      <c r="U181" t="inlineStr">
+        <is>
+          <t>04/10/2026 23:55</t>
+        </is>
+      </c>
       <c r="V181" t="inlineStr">
         <is>
-          <t>⏳ Esperando respuesta</t>
+          <t>🗑️ En destrucción</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-JL037: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -13848,7 +13848,11 @@
         <v>46342</v>
       </c>
       <c r="J193" t="inlineStr"/>
-      <c r="K193" t="inlineStr"/>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="L193" t="inlineStr"/>
       <c r="M193" t="inlineStr"/>
       <c r="N193" t="inlineStr"/>
@@ -13864,10 +13868,14 @@
       <c r="R193" t="inlineStr"/>
       <c r="S193" t="inlineStr"/>
       <c r="T193" t="inlineStr"/>
-      <c r="U193" t="inlineStr"/>
+      <c r="U193" t="inlineStr">
+        <is>
+          <t>05/10/2026 00:29</t>
+        </is>
+      </c>
       <c r="V193" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>🚚 En recolección</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-AG033: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -15508,7 +15508,11 @@
         <v>46372</v>
       </c>
       <c r="J220" t="inlineStr"/>
-      <c r="K220" t="inlineStr"/>
+      <c r="K220" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="L220" t="inlineStr"/>
       <c r="M220" t="inlineStr"/>
       <c r="N220" t="inlineStr"/>
@@ -15524,10 +15528,14 @@
       <c r="R220" t="inlineStr"/>
       <c r="S220" t="inlineStr"/>
       <c r="T220" t="inlineStr"/>
-      <c r="U220" t="inlineStr"/>
+      <c r="U220" t="inlineStr">
+        <is>
+          <t>05/10/2026 00:31</t>
+        </is>
+      </c>
       <c r="V220" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>🚚 En recolección</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-JN027: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -10118,10 +10118,14 @@
       <c r="R135" t="inlineStr"/>
       <c r="S135" t="inlineStr"/>
       <c r="T135" t="inlineStr"/>
-      <c r="U135" t="inlineStr"/>
+      <c r="U135" t="inlineStr">
+        <is>
+          <t>05/10/2026 00:32</t>
+        </is>
+      </c>
       <c r="V135" t="inlineStr">
         <is>
-          <t>🗑️ En destrucción</t>
+          <t>🚚 En recolección</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-JL040: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -12856,7 +12856,11 @@
         <v>46342</v>
       </c>
       <c r="J177" t="inlineStr"/>
-      <c r="K177" t="inlineStr"/>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="L177" t="inlineStr"/>
       <c r="M177" t="inlineStr"/>
       <c r="N177" t="inlineStr"/>
@@ -12872,10 +12876,14 @@
       <c r="R177" t="inlineStr"/>
       <c r="S177" t="inlineStr"/>
       <c r="T177" t="inlineStr"/>
-      <c r="U177" t="inlineStr"/>
+      <c r="U177" t="inlineStr">
+        <is>
+          <t>05/10/2026 00:36</t>
+        </is>
+      </c>
       <c r="V177" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>🚚 En recolección</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-AG035: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -16636,7 +16636,11 @@
         <v>46372</v>
       </c>
       <c r="J238" t="inlineStr"/>
-      <c r="K238" t="inlineStr"/>
+      <c r="K238" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="L238" t="inlineStr"/>
       <c r="M238" t="inlineStr"/>
       <c r="N238" t="inlineStr"/>
@@ -16652,10 +16656,14 @@
       <c r="R238" t="inlineStr"/>
       <c r="S238" t="inlineStr"/>
       <c r="T238" t="inlineStr"/>
-      <c r="U238" t="inlineStr"/>
+      <c r="U238" t="inlineStr">
+        <is>
+          <t>05/10/2026 00:37</t>
+        </is>
+      </c>
       <c r="V238" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>🚚 En recolección</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-JL050: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -11981,12 +11981,16 @@
           <t>Recolección</t>
         </is>
       </c>
-      <c r="L163" t="inlineStr"/>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>8425</t>
+        </is>
+      </c>
       <c r="M163" t="inlineStr"/>
       <c r="N163" t="inlineStr"/>
       <c r="O163" t="inlineStr">
         <is>
-          <t>[25/08/2026 08:33 · Francisco] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [25/08/2026 08:55 · Francisco] Etapa 2 TERMINADA · Recolección → pasa a Disposición final | [29/08/2026 13:06 · Francisco] Etapa Disposición final TERMINADA → pasa a Cuentas por pagar | [01/09/2026 10:14 · yolanda] Avance en Cuentas por pagar</t>
+          <t>8425</t>
         </is>
       </c>
       <c r="P163" s="1" t="n">
@@ -12000,7 +12004,11 @@
       <c r="R163" t="inlineStr"/>
       <c r="S163" t="inlineStr"/>
       <c r="T163" t="inlineStr"/>
-      <c r="U163" t="inlineStr"/>
+      <c r="U163" t="inlineStr">
+        <is>
+          <t>05/10/2026 00:49</t>
+        </is>
+      </c>
       <c r="V163" t="inlineStr">
         <is>
           <t>📨 Enviado a Cuentas por Pagar</t>

</xml_diff>

<commit_message>
Garantía DC-AG011: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -14004,11 +14004,23 @@
         <v>46372</v>
       </c>
       <c r="J195" t="inlineStr"/>
-      <c r="K195" t="inlineStr"/>
-      <c r="L195" t="inlineStr"/>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>8448</t>
+        </is>
+      </c>
       <c r="M195" t="inlineStr"/>
       <c r="N195" t="inlineStr"/>
-      <c r="O195" t="inlineStr"/>
+      <c r="O195" t="inlineStr">
+        <is>
+          <t>8448 Devolucion</t>
+        </is>
+      </c>
       <c r="P195" s="1" t="n">
         <v>46282</v>
       </c>
@@ -14020,10 +14032,14 @@
       <c r="R195" t="inlineStr"/>
       <c r="S195" t="inlineStr"/>
       <c r="T195" t="inlineStr"/>
-      <c r="U195" t="inlineStr"/>
+      <c r="U195" t="inlineStr">
+        <is>
+          <t>05/10/2026 00:52</t>
+        </is>
+      </c>
       <c r="V195" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-JL011: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -11210,11 +11210,23 @@
         <v>46342</v>
       </c>
       <c r="J151" t="inlineStr"/>
-      <c r="K151" t="inlineStr"/>
-      <c r="L151" t="inlineStr"/>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>8450</t>
+        </is>
+      </c>
       <c r="M151" t="inlineStr"/>
       <c r="N151" t="inlineStr"/>
-      <c r="O151" t="inlineStr"/>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>8450 Devolucion</t>
+        </is>
+      </c>
       <c r="P151" s="1" t="n">
         <v>46252</v>
       </c>
@@ -11226,10 +11238,14 @@
       <c r="R151" t="inlineStr"/>
       <c r="S151" t="inlineStr"/>
       <c r="T151" t="inlineStr"/>
-      <c r="U151" t="inlineStr"/>
+      <c r="U151" t="inlineStr">
+        <is>
+          <t>05/10/2026 01:05</t>
+        </is>
+      </c>
       <c r="V151" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-AG012: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -15928,11 +15928,23 @@
         <v>46372</v>
       </c>
       <c r="J226" t="inlineStr"/>
-      <c r="K226" t="inlineStr"/>
-      <c r="L226" t="inlineStr"/>
+      <c r="K226" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L226" t="inlineStr">
+        <is>
+          <t>8450</t>
+        </is>
+      </c>
       <c r="M226" t="inlineStr"/>
       <c r="N226" t="inlineStr"/>
-      <c r="O226" t="inlineStr"/>
+      <c r="O226" t="inlineStr">
+        <is>
+          <t>8450 Devolucion</t>
+        </is>
+      </c>
       <c r="P226" s="1" t="n">
         <v>46282</v>
       </c>
@@ -15944,10 +15956,14 @@
       <c r="R226" t="inlineStr"/>
       <c r="S226" t="inlineStr"/>
       <c r="T226" t="inlineStr"/>
-      <c r="U226" t="inlineStr"/>
+      <c r="U226" t="inlineStr">
+        <is>
+          <t>05/10/2026 01:06</t>
+        </is>
+      </c>
       <c r="V226" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cuarentena: 1 folio(s) de CHAPA INDUSTRIAS  SA DE CV liberados (DC-JL008)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -11626,11 +11626,11 @@
       <c r="N157" t="inlineStr"/>
       <c r="O157" t="inlineStr"/>
       <c r="P157" s="1" t="n">
-        <v>46252</v>
+        <v>46300</v>
       </c>
       <c r="Q157" t="inlineStr">
         <is>
-          <t>Cuarentena</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="R157" s="1" t="n">
@@ -11640,7 +11640,11 @@
         <v>46316</v>
       </c>
       <c r="T157" t="inlineStr"/>
-      <c r="U157" t="inlineStr"/>
+      <c r="U157" t="inlineStr">
+        <is>
+          <t>05/10/2026 02:00</t>
+        </is>
+      </c>
       <c r="V157" t="inlineStr"/>
     </row>
     <row r="158">

</xml_diff>

<commit_message>
Garantía DC-JL008: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -11620,11 +11620,23 @@
         <v>46342</v>
       </c>
       <c r="J157" t="inlineStr"/>
-      <c r="K157" t="inlineStr"/>
-      <c r="L157" t="inlineStr"/>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>8435</t>
+        </is>
+      </c>
       <c r="M157" t="inlineStr"/>
       <c r="N157" t="inlineStr"/>
-      <c r="O157" t="inlineStr"/>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t>8435 Devolucion</t>
+        </is>
+      </c>
       <c r="P157" s="1" t="n">
         <v>46300</v>
       </c>
@@ -11642,10 +11654,14 @@
       <c r="T157" t="inlineStr"/>
       <c r="U157" t="inlineStr">
         <is>
-          <t>05/10/2026 02:00</t>
-        </is>
-      </c>
-      <c r="V157" t="inlineStr"/>
+          <t>05/10/2026 02:02</t>
+        </is>
+      </c>
+      <c r="V157" t="inlineStr">
+        <is>
+          <t>📨 Enviado a Cuentas por Pagar</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="n">

</xml_diff>

<commit_message>
Cuarentena: 1 folio(s) de CHAPA INDUSTRIAS  SA DE CV liberados (DC-AB023)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -5610,11 +5610,11 @@
         </is>
       </c>
       <c r="P72" s="1" t="n">
-        <v>46162</v>
+        <v>46300</v>
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>Cuarentena</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="R72" s="1" t="n">
@@ -5624,7 +5624,11 @@
         <v>46316</v>
       </c>
       <c r="T72" t="inlineStr"/>
-      <c r="U72" t="inlineStr"/>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>05/10/2026 02:05</t>
+        </is>
+      </c>
       <c r="V72" t="inlineStr"/>
     </row>
     <row r="73">

</xml_diff>

<commit_message>
Garantía DC-AB023: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -5600,7 +5600,11 @@
       <c r="J72" t="n">
         <v>36</v>
       </c>
-      <c r="K72" t="inlineStr"/>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="L72" t="inlineStr"/>
       <c r="M72" t="inlineStr"/>
       <c r="N72" t="inlineStr"/>
@@ -5626,10 +5630,14 @@
       <c r="T72" t="inlineStr"/>
       <c r="U72" t="inlineStr">
         <is>
-          <t>05/10/2026 02:05</t>
-        </is>
-      </c>
-      <c r="V72" t="inlineStr"/>
+          <t>05/10/2026 02:06</t>
+        </is>
+      </c>
+      <c r="V72" t="inlineStr">
+        <is>
+          <t>🚚 En recolección</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">

</xml_diff>

<commit_message>
Garantía DC-AG010: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -14128,7 +14128,11 @@
         <v>46372</v>
       </c>
       <c r="J196" t="inlineStr"/>
-      <c r="K196" t="inlineStr"/>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="L196" t="inlineStr"/>
       <c r="M196" t="inlineStr"/>
       <c r="N196" t="inlineStr"/>
@@ -14144,10 +14148,14 @@
       <c r="R196" t="inlineStr"/>
       <c r="S196" t="inlineStr"/>
       <c r="T196" t="inlineStr"/>
-      <c r="U196" t="inlineStr"/>
+      <c r="U196" t="inlineStr">
+        <is>
+          <t>05/10/2026 02:08</t>
+        </is>
+      </c>
       <c r="V196" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>🚚 En recolección</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-MZ038: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -3187,7 +3187,11 @@
           <t>Recolección</t>
         </is>
       </c>
-      <c r="L39" t="inlineStr"/>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>8463</t>
+        </is>
+      </c>
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr"/>
       <c r="O39" t="inlineStr">
@@ -3206,10 +3210,14 @@
       <c r="R39" t="inlineStr"/>
       <c r="S39" t="inlineStr"/>
       <c r="T39" t="inlineStr"/>
-      <c r="U39" t="inlineStr"/>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>05/10/2026 02:14</t>
+        </is>
+      </c>
       <c r="V39" t="inlineStr">
         <is>
-          <t>🗑️ En destrucción</t>
+          <t>🚚 En recolección</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-JL047: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -11102,7 +11102,11 @@
         <v>46342</v>
       </c>
       <c r="J149" t="inlineStr"/>
-      <c r="K149" t="inlineStr"/>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="L149" t="inlineStr"/>
       <c r="M149" t="inlineStr"/>
       <c r="N149" t="inlineStr"/>
@@ -11118,10 +11122,14 @@
       <c r="R149" t="inlineStr"/>
       <c r="S149" t="inlineStr"/>
       <c r="T149" t="inlineStr"/>
-      <c r="U149" t="inlineStr"/>
+      <c r="U149" t="inlineStr">
+        <is>
+          <t>05/10/2026 02:19</t>
+        </is>
+      </c>
       <c r="V149" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>🚚 En recolección</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-AG039: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -15496,7 +15496,11 @@
         <v>46372</v>
       </c>
       <c r="J218" t="inlineStr"/>
-      <c r="K218" t="inlineStr"/>
+      <c r="K218" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="L218" t="inlineStr"/>
       <c r="M218" t="inlineStr"/>
       <c r="N218" t="inlineStr"/>
@@ -15512,10 +15516,14 @@
       <c r="R218" t="inlineStr"/>
       <c r="S218" t="inlineStr"/>
       <c r="T218" t="inlineStr"/>
-      <c r="U218" t="inlineStr"/>
+      <c r="U218" t="inlineStr">
+        <is>
+          <t>05/10/2026 02:20</t>
+        </is>
+      </c>
       <c r="V218" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>🚚 En recolección</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-AB009: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -4570,10 +4570,14 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>Sin respuesta</t>
-        </is>
-      </c>
-      <c r="L58" t="inlineStr"/>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>8429</t>
+        </is>
+      </c>
       <c r="M58" t="inlineStr"/>
       <c r="N58" t="inlineStr"/>
       <c r="O58" t="inlineStr">
@@ -4592,7 +4596,11 @@
       <c r="R58" t="inlineStr"/>
       <c r="S58" t="inlineStr"/>
       <c r="T58" t="inlineStr"/>
-      <c r="U58" t="inlineStr"/>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>05/10/2026 02:24</t>
+        </is>
+      </c>
       <c r="V58" t="inlineStr">
         <is>
           <t>📨 Enviado a Cuentas por Pagar</t>

</xml_diff>

<commit_message>
Garantía DC-MY024: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -7617,7 +7617,11 @@
           <t>Recolección</t>
         </is>
       </c>
-      <c r="L100" t="inlineStr"/>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>8429</t>
+        </is>
+      </c>
       <c r="M100" t="inlineStr"/>
       <c r="N100" t="inlineStr"/>
       <c r="O100" t="inlineStr">
@@ -7636,7 +7640,11 @@
       <c r="R100" t="inlineStr"/>
       <c r="S100" t="inlineStr"/>
       <c r="T100" t="inlineStr"/>
-      <c r="U100" t="inlineStr"/>
+      <c r="U100" t="inlineStr">
+        <is>
+          <t>05/10/2026 02:25</t>
+        </is>
+      </c>
       <c r="V100" t="inlineStr">
         <is>
           <t>📨 Enviado a Cuentas por Pagar</t>

</xml_diff>

<commit_message>
Garantía DC-JN015: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -9551,7 +9551,11 @@
           <t>Recolección</t>
         </is>
       </c>
-      <c r="L127" t="inlineStr"/>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>8429</t>
+        </is>
+      </c>
       <c r="M127" t="inlineStr"/>
       <c r="N127" t="inlineStr"/>
       <c r="O127" t="inlineStr">
@@ -9570,7 +9574,11 @@
       <c r="R127" t="inlineStr"/>
       <c r="S127" t="inlineStr"/>
       <c r="T127" t="inlineStr"/>
-      <c r="U127" t="inlineStr"/>
+      <c r="U127" t="inlineStr">
+        <is>
+          <t>05/10/2026 02:27</t>
+        </is>
+      </c>
       <c r="V127" t="inlineStr">
         <is>
           <t>📨 Enviado a Cuentas por Pagar</t>

</xml_diff>

<commit_message>
Garantía DC-JL021: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -13893,12 +13893,16 @@
           <t>Recolección</t>
         </is>
       </c>
-      <c r="L192" t="inlineStr"/>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>8429</t>
+        </is>
+      </c>
       <c r="M192" t="inlineStr"/>
       <c r="N192" t="inlineStr"/>
       <c r="O192" t="inlineStr">
         <is>
-          <t>[01/09/2026 10:11 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/09/2026 10:12 · yolanda] Etapa 2 TERMINADA · Recolección → pasa a Disposición final | [01/09/2026 10:13 · yolanda] Etapa Disposición final TERMINADA → pasa a Cuentas por pagar</t>
+          <t>8429 Devolucion</t>
         </is>
       </c>
       <c r="P192" s="1" t="n">
@@ -13912,7 +13916,11 @@
       <c r="R192" t="inlineStr"/>
       <c r="S192" t="inlineStr"/>
       <c r="T192" t="inlineStr"/>
-      <c r="U192" t="inlineStr"/>
+      <c r="U192" t="inlineStr">
+        <is>
+          <t>05/10/2026 02:27</t>
+        </is>
+      </c>
       <c r="V192" t="inlineStr">
         <is>
           <t>📨 Enviado a Cuentas por Pagar</t>

</xml_diff>

<commit_message>
Garantía DC-AG021: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -15212,7 +15212,11 @@
         <v>46372</v>
       </c>
       <c r="J213" t="inlineStr"/>
-      <c r="K213" t="inlineStr"/>
+      <c r="K213" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="L213" t="inlineStr"/>
       <c r="M213" t="inlineStr"/>
       <c r="N213" t="inlineStr"/>
@@ -15228,10 +15232,14 @@
       <c r="R213" t="inlineStr"/>
       <c r="S213" t="inlineStr"/>
       <c r="T213" t="inlineStr"/>
-      <c r="U213" t="inlineStr"/>
+      <c r="U213" t="inlineStr">
+        <is>
+          <t>05/10/2026 02:28</t>
+        </is>
+      </c>
       <c r="V213" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>🚚 En recolección</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-JL052: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -12321,10 +12321,18 @@
       </c>
       <c r="J167" t="inlineStr"/>
       <c r="K167" t="inlineStr"/>
-      <c r="L167" t="inlineStr"/>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>8439</t>
+        </is>
+      </c>
       <c r="M167" t="inlineStr"/>
       <c r="N167" t="inlineStr"/>
-      <c r="O167" t="inlineStr"/>
+      <c r="O167" t="inlineStr">
+        <is>
+          <t>8439 Devolucion</t>
+        </is>
+      </c>
       <c r="P167" s="1" t="n">
         <v>46252</v>
       </c>
@@ -12336,10 +12344,14 @@
       <c r="R167" t="inlineStr"/>
       <c r="S167" t="inlineStr"/>
       <c r="T167" t="inlineStr"/>
-      <c r="U167" t="inlineStr"/>
+      <c r="U167" t="inlineStr">
+        <is>
+          <t>05/10/2026 02:31</t>
+        </is>
+      </c>
       <c r="V167" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-JN008: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -9191,12 +9191,16 @@
           <t>Recolección</t>
         </is>
       </c>
-      <c r="L122" t="inlineStr"/>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>8444</t>
+        </is>
+      </c>
       <c r="M122" t="inlineStr"/>
       <c r="N122" t="inlineStr"/>
       <c r="O122" t="inlineStr">
         <is>
-          <t>DEVOLUCION</t>
+          <t>8444   DEVOLUCION</t>
         </is>
       </c>
       <c r="P122" s="1" t="n">
@@ -9210,10 +9214,14 @@
       <c r="R122" t="inlineStr"/>
       <c r="S122" t="inlineStr"/>
       <c r="T122" t="inlineStr"/>
-      <c r="U122" t="inlineStr"/>
+      <c r="U122" t="inlineStr">
+        <is>
+          <t>05/10/2026 02:38</t>
+        </is>
+      </c>
       <c r="V122" t="inlineStr">
         <is>
-          <t>🗑️ En destrucción</t>
+          <t>📄 Folio devolución/ajuste generado</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-JL014: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -12012,8 +12012,16 @@
         <v>46342</v>
       </c>
       <c r="J162" t="inlineStr"/>
-      <c r="K162" t="inlineStr"/>
-      <c r="L162" t="inlineStr"/>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>8444</t>
+        </is>
+      </c>
       <c r="M162" t="inlineStr"/>
       <c r="N162" t="inlineStr"/>
       <c r="O162" t="inlineStr"/>
@@ -12028,10 +12036,14 @@
       <c r="R162" t="inlineStr"/>
       <c r="S162" t="inlineStr"/>
       <c r="T162" t="inlineStr"/>
-      <c r="U162" t="inlineStr"/>
+      <c r="U162" t="inlineStr">
+        <is>
+          <t>05/10/2026 02:41</t>
+        </is>
+      </c>
       <c r="V162" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cuarentena: 1 folio(s) de KWIKSET RESIDENCIAL MEXICO SA DE CV liberados (DC-AB014)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -4954,11 +4954,11 @@
         </is>
       </c>
       <c r="P63" s="1" t="n">
-        <v>46162</v>
+        <v>46300</v>
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>Cuarentena</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="R63" s="1" t="n">
@@ -4968,7 +4968,11 @@
         <v>46316</v>
       </c>
       <c r="T63" t="inlineStr"/>
-      <c r="U63" t="inlineStr"/>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>05/10/2026 08:40</t>
+        </is>
+      </c>
       <c r="V63" t="inlineStr"/>
     </row>
     <row r="64">

</xml_diff>

<commit_message>
Garantía DC-AB014: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -4945,12 +4945,16 @@
           <t>Recolección</t>
         </is>
       </c>
-      <c r="L63" t="inlineStr"/>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>8282</t>
+        </is>
+      </c>
       <c r="M63" t="inlineStr"/>
       <c r="N63" t="inlineStr"/>
       <c r="O63" t="inlineStr">
         <is>
-          <t>DEVOLUCION</t>
+          <t>8282 DEVOLUCION</t>
         </is>
       </c>
       <c r="P63" s="1" t="n">
@@ -4970,10 +4974,14 @@
       <c r="T63" t="inlineStr"/>
       <c r="U63" t="inlineStr">
         <is>
-          <t>05/10/2026 08:40</t>
-        </is>
-      </c>
-      <c r="V63" t="inlineStr"/>
+          <t>05/10/2026 08:41</t>
+        </is>
+      </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>📨 Enviado a Cuentas por Pagar</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">

</xml_diff>

<commit_message>
Garantía DC-MZ017: Folio marcado como RESUELTO (fecha cierre 05/10/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1705,7 +1705,11 @@
         </is>
       </c>
       <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>173952</t>
+        </is>
+      </c>
       <c r="O18" t="inlineStr">
         <is>
           <t>DEVOLUCION</t>
@@ -1716,7 +1720,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R18" s="1" t="n">
@@ -1725,10 +1729,12 @@
       <c r="S18" s="1" t="n">
         <v>46316</v>
       </c>
-      <c r="T18" t="inlineStr"/>
+      <c r="T18" s="1" t="n">
+        <v>46300</v>
+      </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>28/09/2026 11:41</t>
+          <t>05/10/2026 12:55</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">

</xml_diff>

<commit_message>
Garantía DC-JL050: Folio marcado como RESUELTO (fecha cierre 05/10/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -12113,7 +12113,11 @@
         </is>
       </c>
       <c r="M163" t="inlineStr"/>
-      <c r="N163" t="inlineStr"/>
+      <c r="N163" t="inlineStr">
+        <is>
+          <t>174864</t>
+        </is>
+      </c>
       <c r="O163" t="inlineStr">
         <is>
           <t>8425</t>
@@ -12124,15 +12128,17 @@
       </c>
       <c r="Q163" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R163" t="inlineStr"/>
       <c r="S163" t="inlineStr"/>
-      <c r="T163" t="inlineStr"/>
+      <c r="T163" s="1" t="n">
+        <v>46300</v>
+      </c>
       <c r="U163" t="inlineStr">
         <is>
-          <t>05/10/2026 00:49</t>
+          <t>05/10/2026 13:00</t>
         </is>
       </c>
       <c r="V163" t="inlineStr">

</xml_diff>

<commit_message>
Garantía DC-JL048: Folio marcado como RESUELTO (fecha cierre 05/10/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -12575,22 +12575,28 @@
         </is>
       </c>
       <c r="M170" t="inlineStr"/>
-      <c r="N170" t="inlineStr"/>
+      <c r="N170" t="inlineStr">
+        <is>
+          <t>486230</t>
+        </is>
+      </c>
       <c r="O170" t="inlineStr"/>
       <c r="P170" s="1" t="n">
         <v>46252</v>
       </c>
       <c r="Q170" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R170" t="inlineStr"/>
       <c r="S170" t="inlineStr"/>
-      <c r="T170" t="inlineStr"/>
+      <c r="T170" s="1" t="n">
+        <v>46300</v>
+      </c>
       <c r="U170" t="inlineStr">
         <is>
-          <t>28/09/2026 13:10</t>
+          <t>05/10/2026 13:02</t>
         </is>
       </c>
       <c r="V170" t="inlineStr">

</xml_diff>

<commit_message>
Garantía DC-MZ030: Folio marcado como RESUELTO (fecha cierre 30/09/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -2633,7 +2633,11 @@
         </is>
       </c>
       <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>176113</t>
+        </is>
+      </c>
       <c r="O31" t="inlineStr">
         <is>
           <t>DEVOLUCION</t>
@@ -2644,15 +2648,17 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R31" t="inlineStr"/>
       <c r="S31" t="inlineStr"/>
-      <c r="T31" t="inlineStr"/>
+      <c r="T31" s="1" t="n">
+        <v>46295</v>
+      </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>28/09/2026 11:45</t>
+          <t>05/10/2026 17:04</t>
         </is>
       </c>
       <c r="V31" t="inlineStr">

</xml_diff>

<commit_message>
Garantía DC-AB014: Folio marcado como RESUELTO (fecha cierre 15/09/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -4963,7 +4963,11 @@
         </is>
       </c>
       <c r="M63" t="inlineStr"/>
-      <c r="N63" t="inlineStr"/>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>48812</t>
+        </is>
+      </c>
       <c r="O63" t="inlineStr">
         <is>
           <t>8282 DEVOLUCION</t>
@@ -4974,7 +4978,7 @@
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R63" s="1" t="n">
@@ -4983,10 +4987,12 @@
       <c r="S63" s="1" t="n">
         <v>46316</v>
       </c>
-      <c r="T63" t="inlineStr"/>
+      <c r="T63" s="1" t="n">
+        <v>46280</v>
+      </c>
       <c r="U63" t="inlineStr">
         <is>
-          <t>05/10/2026 08:41</t>
+          <t>05/10/2026 17:41</t>
         </is>
       </c>
       <c r="V63" t="inlineStr">

</xml_diff>

<commit_message>
Garantía DC-JN028: Folio marcado como RESUELTO (fecha cierre 11/09/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -10257,7 +10257,11 @@
       </c>
       <c r="L136" t="inlineStr"/>
       <c r="M136" t="inlineStr"/>
-      <c r="N136" t="inlineStr"/>
+      <c r="N136" t="inlineStr">
+        <is>
+          <t>224226</t>
+        </is>
+      </c>
       <c r="O136" t="inlineStr">
         <is>
           <t>DESTRUCCION  RM-30496035</t>
@@ -10268,7 +10272,7 @@
       </c>
       <c r="Q136" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R136" s="1" t="n">
@@ -10277,10 +10281,12 @@
       <c r="S136" s="1" t="n">
         <v>46316</v>
       </c>
-      <c r="T136" t="inlineStr"/>
+      <c r="T136" s="1" t="n">
+        <v>46276</v>
+      </c>
       <c r="U136" t="inlineStr">
         <is>
-          <t>03/10/2026 12:22</t>
+          <t>05/10/2026 17:56</t>
         </is>
       </c>
       <c r="V136" t="inlineStr">

</xml_diff>

<commit_message>
Garantía DC-JL038: Folio marcado como RESUELTO (fecha cierre 05/10/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -11029,7 +11029,11 @@
       </c>
       <c r="L147" t="inlineStr"/>
       <c r="M147" t="inlineStr"/>
-      <c r="N147" t="inlineStr"/>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>224226</t>
+        </is>
+      </c>
       <c r="O147" t="inlineStr">
         <is>
           <t>nc -DM30496035</t>
@@ -11040,15 +11044,17 @@
       </c>
       <c r="Q147" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R147" t="inlineStr"/>
       <c r="S147" t="inlineStr"/>
-      <c r="T147" t="inlineStr"/>
+      <c r="T147" s="1" t="n">
+        <v>46300</v>
+      </c>
       <c r="U147" t="inlineStr">
         <is>
-          <t>03/10/2026 12:19</t>
+          <t>05/10/2026 18:01</t>
         </is>
       </c>
       <c r="V147" t="inlineStr">

</xml_diff>

<commit_message>
Garantía DC-AB038: Folio marcado como RESUELTO (fecha cierre 11/08/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -6509,7 +6509,11 @@
         </is>
       </c>
       <c r="M84" t="inlineStr"/>
-      <c r="N84" t="inlineStr"/>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>174123</t>
+        </is>
+      </c>
       <c r="O84" t="inlineStr">
         <is>
           <t>DEVOLUCION 8359 | [01/09/2026 08:50 · Yolanda Jeronimo] Avance en Cuentas por pagar | [01/09/2026 08:51 · yolanda] Avance en Cuentas por pagar | [01/09/2026 08:53 · Yolanda Jeronimo] Avance en Cuentas por pagar | [01/09/2026 08:57 · Yolanda Jeronimo] Avance en Cuentas por pagar | [01/09/2026 09:10 · Admin cuarentena] 1 reclamación(es) de INTERRUPTORES Y GABINETES ELECTRICOS SA DE CV liberadas de cuarentena → Reporte de reclamo</t>
@@ -6520,7 +6524,7 @@
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R84" s="1" t="n">
@@ -6529,10 +6533,12 @@
       <c r="S84" s="1" t="n">
         <v>46316</v>
       </c>
-      <c r="T84" t="inlineStr"/>
+      <c r="T84" s="1" t="n">
+        <v>46245</v>
+      </c>
       <c r="U84" t="inlineStr">
         <is>
-          <t>28/09/2026 13:01</t>
+          <t>05/10/2026 18:11</t>
         </is>
       </c>
       <c r="V84" t="inlineStr">

</xml_diff>

<commit_message>
Garantía DC-AB005: Folio marcado como RESUELTO (fecha cierre 09/10/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -4303,7 +4303,11 @@
         </is>
       </c>
       <c r="M54" t="inlineStr"/>
-      <c r="N54" t="inlineStr"/>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>49261</t>
+        </is>
+      </c>
       <c r="O54" t="inlineStr">
         <is>
           <t>DEVOLUCION 8375</t>
@@ -4314,13 +4318,19 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R54" t="inlineStr"/>
       <c r="S54" t="inlineStr"/>
-      <c r="T54" t="inlineStr"/>
-      <c r="U54" t="inlineStr"/>
+      <c r="T54" s="1" t="n">
+        <v>46304</v>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>11/10/2026 19:04</t>
+        </is>
+      </c>
       <c r="V54" t="inlineStr">
         <is>
           <t>📨 Enviado a Cuentas por Pagar</t>

</xml_diff>

<commit_message>
Garantía DC-MY018: Folio marcado como RESUELTO (fecha cierre 09/10/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -7467,7 +7467,11 @@
         </is>
       </c>
       <c r="M97" t="inlineStr"/>
-      <c r="N97" t="inlineStr"/>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>49261</t>
+        </is>
+      </c>
       <c r="O97" t="inlineStr">
         <is>
           <t>DEVOLUCION 8375</t>
@@ -7478,13 +7482,19 @@
       </c>
       <c r="Q97" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R97" t="inlineStr"/>
       <c r="S97" t="inlineStr"/>
-      <c r="T97" t="inlineStr"/>
-      <c r="U97" t="inlineStr"/>
+      <c r="T97" s="1" t="n">
+        <v>46304</v>
+      </c>
+      <c r="U97" t="inlineStr">
+        <is>
+          <t>11/10/2026 19:04</t>
+        </is>
+      </c>
       <c r="V97" t="inlineStr">
         <is>
           <t>📨 Enviado a Cuentas por Pagar</t>

</xml_diff>

<commit_message>
Garantía DC-JL012: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -13609,7 +13609,11 @@
         <v>38</v>
       </c>
       <c r="K184" t="inlineStr"/>
-      <c r="L184" t="inlineStr"/>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>8465</t>
+        </is>
+      </c>
       <c r="M184" t="inlineStr"/>
       <c r="N184" t="inlineStr"/>
       <c r="O184" t="inlineStr"/>
@@ -13624,7 +13628,11 @@
       <c r="R184" t="inlineStr"/>
       <c r="S184" t="inlineStr"/>
       <c r="T184" t="inlineStr"/>
-      <c r="U184" t="inlineStr"/>
+      <c r="U184" t="inlineStr">
+        <is>
+          <t>11/10/2026 20:23</t>
+        </is>
+      </c>
       <c r="V184" t="inlineStr">
         <is>
           <t>📝 Reporte recibido</t>

</xml_diff>

<commit_message>
Garantía DC-JN037: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -19844,8 +19844,16 @@
       <c r="J281" t="n">
         <v>91</v>
       </c>
-      <c r="K281" t="inlineStr"/>
-      <c r="L281" t="inlineStr"/>
+      <c r="K281" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L281" t="inlineStr">
+        <is>
+          <t>8469</t>
+        </is>
+      </c>
       <c r="M281" t="inlineStr"/>
       <c r="N281" t="inlineStr"/>
       <c r="O281" t="inlineStr"/>
@@ -19860,10 +19868,14 @@
       <c r="R281" t="inlineStr"/>
       <c r="S281" t="inlineStr"/>
       <c r="T281" t="inlineStr"/>
-      <c r="U281" t="inlineStr"/>
+      <c r="U281" t="inlineStr">
+        <is>
+          <t>11/10/2026 21:54</t>
+        </is>
+      </c>
       <c r="V281" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Casos especiales: + FERREMOVIL DEL NORTE SA DE CV (Otro motivo)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -33577,7 +33577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33622,6 +33622,26 @@
         <v>46297</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FERREMOVIL DEL NORTE SA DE CV</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Otro motivo</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>PROVEEDOR   SE HACE ORDEN DE COMPRA Y PEDIDO SE ENTREGA EN 6 MESES</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>46306</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Garantía DC-MY013: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -17984,8 +17984,16 @@
       <c r="J251" t="n">
         <v>91</v>
       </c>
-      <c r="K251" t="inlineStr"/>
-      <c r="L251" t="inlineStr"/>
+      <c r="K251" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L251" t="inlineStr">
+        <is>
+          <t>8361</t>
+        </is>
+      </c>
       <c r="M251" t="inlineStr"/>
       <c r="N251" t="inlineStr"/>
       <c r="O251" t="inlineStr"/>
@@ -18000,10 +18008,14 @@
       <c r="R251" t="inlineStr"/>
       <c r="S251" t="inlineStr"/>
       <c r="T251" t="inlineStr"/>
-      <c r="U251" t="inlineStr"/>
+      <c r="U251" t="inlineStr">
+        <is>
+          <t>12/10/2026 09:21</t>
+        </is>
+      </c>
       <c r="V251" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-JN007: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -19298,8 +19298,16 @@
       <c r="J272" t="n">
         <v>91</v>
       </c>
-      <c r="K272" t="inlineStr"/>
-      <c r="L272" t="inlineStr"/>
+      <c r="K272" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L272" t="inlineStr">
+        <is>
+          <t>8450</t>
+        </is>
+      </c>
       <c r="M272" t="inlineStr"/>
       <c r="N272" t="inlineStr"/>
       <c r="O272" t="inlineStr"/>
@@ -19314,10 +19322,14 @@
       <c r="R272" t="inlineStr"/>
       <c r="S272" t="inlineStr"/>
       <c r="T272" t="inlineStr"/>
-      <c r="U272" t="inlineStr"/>
+      <c r="U272" t="inlineStr">
+        <is>
+          <t>12/10/2026 09:22</t>
+        </is>
+      </c>
       <c r="V272" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-MZ010: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1215,7 +1215,11 @@
           <t>Recolección</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>8392</t>
+        </is>
+      </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr">
@@ -1234,7 +1238,11 @@
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr"/>
-      <c r="U11" t="inlineStr"/>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>12/10/2026 09:35</t>
+        </is>
+      </c>
       <c r="V11" t="inlineStr">
         <is>
           <t>📨 Enviado a Cuentas por Pagar</t>

</xml_diff>

<commit_message>
Garantía DC-MY015: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -7321,7 +7321,11 @@
           <t>Recolección</t>
         </is>
       </c>
-      <c r="L95" t="inlineStr"/>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>8392</t>
+        </is>
+      </c>
       <c r="M95" t="inlineStr"/>
       <c r="N95" t="inlineStr"/>
       <c r="O95" t="inlineStr">
@@ -7340,7 +7344,11 @@
       <c r="R95" t="inlineStr"/>
       <c r="S95" t="inlineStr"/>
       <c r="T95" t="inlineStr"/>
-      <c r="U95" t="inlineStr"/>
+      <c r="U95" t="inlineStr">
+        <is>
+          <t>12/10/2026 09:36</t>
+        </is>
+      </c>
       <c r="V95" t="inlineStr">
         <is>
           <t>📨 Enviado a Cuentas por Pagar</t>

</xml_diff>

<commit_message>
Garantía DC-AG013: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -17938,8 +17938,16 @@
       <c r="J250" t="n">
         <v>68</v>
       </c>
-      <c r="K250" t="inlineStr"/>
-      <c r="L250" t="inlineStr"/>
+      <c r="K250" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L250" t="inlineStr">
+        <is>
+          <t>8465</t>
+        </is>
+      </c>
       <c r="M250" t="inlineStr"/>
       <c r="N250" t="inlineStr"/>
       <c r="O250" t="inlineStr"/>
@@ -17954,10 +17962,14 @@
       <c r="R250" t="inlineStr"/>
       <c r="S250" t="inlineStr"/>
       <c r="T250" t="inlineStr"/>
-      <c r="U250" t="inlineStr"/>
+      <c r="U250" t="inlineStr">
+        <is>
+          <t>12/10/2026 09:40</t>
+        </is>
+      </c>
       <c r="V250" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-MY029: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -18397,7 +18397,11 @@
         <v>91</v>
       </c>
       <c r="K257" t="inlineStr"/>
-      <c r="L257" t="inlineStr"/>
+      <c r="L257" t="inlineStr">
+        <is>
+          <t>8341</t>
+        </is>
+      </c>
       <c r="M257" t="inlineStr"/>
       <c r="N257" t="inlineStr"/>
       <c r="O257" t="inlineStr"/>
@@ -18412,7 +18416,11 @@
       <c r="R257" t="inlineStr"/>
       <c r="S257" t="inlineStr"/>
       <c r="T257" t="inlineStr"/>
-      <c r="U257" t="inlineStr"/>
+      <c r="U257" t="inlineStr">
+        <is>
+          <t>12/10/2026 09:49</t>
+        </is>
+      </c>
       <c r="V257" t="inlineStr">
         <is>
           <t>📝 Reporte recibido</t>

</xml_diff>

<commit_message>
Garantía DC-JN021: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -19537,7 +19537,11 @@
         <v>91</v>
       </c>
       <c r="K275" t="inlineStr"/>
-      <c r="L275" t="inlineStr"/>
+      <c r="L275" t="inlineStr">
+        <is>
+          <t>8341</t>
+        </is>
+      </c>
       <c r="M275" t="inlineStr"/>
       <c r="N275" t="inlineStr"/>
       <c r="O275" t="inlineStr"/>
@@ -19552,7 +19556,11 @@
       <c r="R275" t="inlineStr"/>
       <c r="S275" t="inlineStr"/>
       <c r="T275" t="inlineStr"/>
-      <c r="U275" t="inlineStr"/>
+      <c r="U275" t="inlineStr">
+        <is>
+          <t>12/10/2026 09:51</t>
+        </is>
+      </c>
       <c r="V275" t="inlineStr">
         <is>
           <t>📝 Reporte recibido</t>

</xml_diff>

<commit_message>
Garantía DC-MZ026: Folio marcado como RESUELTO (con NC, fecha cierre 06/10/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -2361,10 +2361,14 @@
         </is>
       </c>
       <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>176319</t>
+        </is>
+      </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>DEVOLUCION 8341</t>
+          <t>DEVOLUCION 8341 descontado en  T-176319  EL 06/10/2026</t>
         </is>
       </c>
       <c r="P27" s="1" t="n">
@@ -2372,13 +2376,19 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr"/>
-      <c r="T27" t="inlineStr"/>
-      <c r="U27" t="inlineStr"/>
+      <c r="T27" s="1" t="n">
+        <v>46301</v>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>12/10/2026 10:02</t>
+        </is>
+      </c>
       <c r="V27" t="inlineStr">
         <is>
           <t>📨 Enviado a Cuentas por Pagar</t>

</xml_diff>

<commit_message>
Garantía DC-AB011: Folio marcado como RESUELTO (con NC, fecha cierre 12/10/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -4777,10 +4777,14 @@
         </is>
       </c>
       <c r="M60" t="inlineStr"/>
-      <c r="N60" t="inlineStr"/>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>176319</t>
+        </is>
+      </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>DEVOLUCION 8341</t>
+          <t>DEVOLUCION 8341   T-176319  EL 06/10/2026</t>
         </is>
       </c>
       <c r="P60" s="1" t="n">
@@ -4788,13 +4792,19 @@
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R60" t="inlineStr"/>
       <c r="S60" t="inlineStr"/>
-      <c r="T60" t="inlineStr"/>
-      <c r="U60" t="inlineStr"/>
+      <c r="T60" s="1" t="n">
+        <v>46307</v>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>12/10/2026 10:03</t>
+        </is>
+      </c>
       <c r="V60" t="inlineStr">
         <is>
           <t>📨 Enviado a Cuentas por Pagar</t>

</xml_diff>

<commit_message>
Cuarentena: 2 folio(s) de MARIBEL CONTRERAS SOTO liberados (DC-MY041, DC-JN030)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -18620,11 +18620,11 @@
       <c r="N260" t="inlineStr"/>
       <c r="O260" t="inlineStr"/>
       <c r="P260" s="1" t="n">
-        <v>46305</v>
+        <v>46307</v>
       </c>
       <c r="Q260" t="inlineStr">
         <is>
-          <t>Cuarentena</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="R260" s="1" t="n">
@@ -18634,7 +18634,11 @@
         <v>46334</v>
       </c>
       <c r="T260" t="inlineStr"/>
-      <c r="U260" t="inlineStr"/>
+      <c r="U260" t="inlineStr">
+        <is>
+          <t>12/10/2026 10:08</t>
+        </is>
+      </c>
       <c r="V260" t="inlineStr"/>
     </row>
     <row r="261">
@@ -19756,11 +19760,11 @@
       <c r="N278" t="inlineStr"/>
       <c r="O278" t="inlineStr"/>
       <c r="P278" s="1" t="n">
-        <v>46305</v>
+        <v>46307</v>
       </c>
       <c r="Q278" t="inlineStr">
         <is>
-          <t>Cuarentena</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="R278" s="1" t="n">
@@ -19770,7 +19774,11 @@
         <v>46334</v>
       </c>
       <c r="T278" t="inlineStr"/>
-      <c r="U278" t="inlineStr"/>
+      <c r="U278" t="inlineStr">
+        <is>
+          <t>12/10/2026 10:08</t>
+        </is>
+      </c>
       <c r="V278" t="inlineStr"/>
     </row>
     <row r="279">

</xml_diff>

<commit_message>
Garantía DC-MY041: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -18614,8 +18614,16 @@
       <c r="J260" t="n">
         <v>91</v>
       </c>
-      <c r="K260" t="inlineStr"/>
-      <c r="L260" t="inlineStr"/>
+      <c r="K260" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L260" t="inlineStr">
+        <is>
+          <t>8440</t>
+        </is>
+      </c>
       <c r="M260" t="inlineStr"/>
       <c r="N260" t="inlineStr"/>
       <c r="O260" t="inlineStr"/>
@@ -18636,10 +18644,14 @@
       <c r="T260" t="inlineStr"/>
       <c r="U260" t="inlineStr">
         <is>
-          <t>12/10/2026 10:08</t>
-        </is>
-      </c>
-      <c r="V260" t="inlineStr"/>
+          <t>12/10/2026 10:09</t>
+        </is>
+      </c>
+      <c r="V260" t="inlineStr">
+        <is>
+          <t>📨 Enviado a Cuentas por Pagar</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="1" t="n">
@@ -19779,7 +19791,11 @@
           <t>12/10/2026 10:08</t>
         </is>
       </c>
-      <c r="V278" t="inlineStr"/>
+      <c r="V278" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="1" t="n">

</xml_diff>

<commit_message>
Garantía DC-JN030: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -19766,8 +19766,16 @@
       <c r="J278" t="n">
         <v>91</v>
       </c>
-      <c r="K278" t="inlineStr"/>
-      <c r="L278" t="inlineStr"/>
+      <c r="K278" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L278" t="inlineStr">
+        <is>
+          <t>8440</t>
+        </is>
+      </c>
       <c r="M278" t="inlineStr"/>
       <c r="N278" t="inlineStr"/>
       <c r="O278" t="inlineStr"/>
@@ -19788,12 +19796,12 @@
       <c r="T278" t="inlineStr"/>
       <c r="U278" t="inlineStr">
         <is>
-          <t>12/10/2026 10:08</t>
+          <t>12/10/2026 10:09</t>
         </is>
       </c>
       <c r="V278" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-AB025: Folio marcado como RESUELTO (con NC, fecha cierre 18/06/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -5846,7 +5846,7 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>Destrucción</t>
+          <t>Recolección</t>
         </is>
       </c>
       <c r="L74" t="inlineStr">
@@ -5855,10 +5855,14 @@
         </is>
       </c>
       <c r="M74" t="inlineStr"/>
-      <c r="N74" t="inlineStr"/>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>171823</t>
+        </is>
+      </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>DESTRUCCION</t>
+          <t>Dev 8307  DESC T/171823 18/06/2026</t>
         </is>
       </c>
       <c r="P74" s="1" t="n">
@@ -5866,15 +5870,17 @@
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R74" t="inlineStr"/>
       <c r="S74" t="inlineStr"/>
-      <c r="T74" t="inlineStr"/>
+      <c r="T74" s="1" t="n">
+        <v>46191</v>
+      </c>
       <c r="U74" t="inlineStr">
         <is>
-          <t>30/09/2026 11:45</t>
+          <t>12/10/2026 10:16</t>
         </is>
       </c>
       <c r="V74" t="inlineStr">

</xml_diff>

<commit_message>
Garantía DC-MY033: Folio marcado como RESUELTO (con NC, fecha cierre 30/09/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -8087,10 +8087,14 @@
         </is>
       </c>
       <c r="M105" t="inlineStr"/>
-      <c r="N105" t="inlineStr"/>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>176113</t>
+        </is>
+      </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>DEVOLUCION</t>
+          <t>DEVOLUCION 8397   DESC.EN T/176113 30/09/2026</t>
         </is>
       </c>
       <c r="P105" s="1" t="n">
@@ -8098,15 +8102,17 @@
       </c>
       <c r="Q105" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R105" t="inlineStr"/>
       <c r="S105" t="inlineStr"/>
-      <c r="T105" t="inlineStr"/>
+      <c r="T105" s="1" t="n">
+        <v>46295</v>
+      </c>
       <c r="U105" t="inlineStr">
         <is>
-          <t>28/09/2026 11:46</t>
+          <t>12/10/2026 10:21</t>
         </is>
       </c>
       <c r="V105" t="inlineStr">

</xml_diff>

<commit_message>
Garantía DC-MY013: Folio marcado como RESUELTO (con NC, fecha cierre 24/07/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -18055,22 +18055,32 @@
         </is>
       </c>
       <c r="M251" t="inlineStr"/>
-      <c r="N251" t="inlineStr"/>
-      <c r="O251" t="inlineStr"/>
+      <c r="N251" t="inlineStr">
+        <is>
+          <t>173426</t>
+        </is>
+      </c>
+      <c r="O251" t="inlineStr">
+        <is>
+          <t>8361   DESC. T/173426 24 JULIO</t>
+        </is>
+      </c>
       <c r="P251" s="1" t="n">
         <v>46305</v>
       </c>
       <c r="Q251" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R251" t="inlineStr"/>
       <c r="S251" t="inlineStr"/>
-      <c r="T251" t="inlineStr"/>
+      <c r="T251" s="1" t="n">
+        <v>46227</v>
+      </c>
       <c r="U251" t="inlineStr">
         <is>
-          <t>12/10/2026 09:21</t>
+          <t>12/10/2026 10:30</t>
         </is>
       </c>
       <c r="V251" t="inlineStr">

</xml_diff>

<commit_message>
Garantía DC-JL053: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -12334,7 +12334,11 @@
       <c r="J164" t="n">
         <v>38</v>
       </c>
-      <c r="K164" t="inlineStr"/>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>Destrucción</t>
+        </is>
+      </c>
       <c r="L164" t="inlineStr"/>
       <c r="M164" t="inlineStr"/>
       <c r="N164" t="inlineStr"/>
@@ -12350,10 +12354,14 @@
       <c r="R164" t="inlineStr"/>
       <c r="S164" t="inlineStr"/>
       <c r="T164" t="inlineStr"/>
-      <c r="U164" t="inlineStr"/>
+      <c r="U164" t="inlineStr">
+        <is>
+          <t>19/10/2026 11:03</t>
+        </is>
+      </c>
       <c r="V164" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cuarentena: 2 folio(s) de MASTERCIM INDUSTRIAL S.A DE C.V liberados (DC-AG050, DC-SEP043)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -15956,11 +15956,11 @@
       <c r="N219" t="inlineStr"/>
       <c r="O219" t="inlineStr"/>
       <c r="P219" s="1" t="n">
-        <v>46282</v>
+        <v>46314</v>
       </c>
       <c r="Q219" t="inlineStr">
         <is>
-          <t>Cuarentena</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="R219" s="1" t="n">
@@ -15970,7 +15970,11 @@
         <v>46316</v>
       </c>
       <c r="T219" t="inlineStr"/>
-      <c r="U219" t="inlineStr"/>
+      <c r="U219" t="inlineStr">
+        <is>
+          <t>19/10/2026 11:03</t>
+        </is>
+      </c>
       <c r="V219" t="inlineStr"/>
     </row>
     <row r="220">
@@ -22868,11 +22872,11 @@
       <c r="N327" t="inlineStr"/>
       <c r="O327" t="inlineStr"/>
       <c r="P327" s="1" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="Q327" t="inlineStr">
         <is>
-          <t>Cuarentena</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="R327" s="1" t="n">
@@ -22882,7 +22886,11 @@
         <v>46343</v>
       </c>
       <c r="T327" t="inlineStr"/>
-      <c r="U327" t="inlineStr"/>
+      <c r="U327" t="inlineStr">
+        <is>
+          <t>19/10/2026 11:03</t>
+        </is>
+      </c>
       <c r="V327" t="inlineStr"/>
     </row>
     <row r="328">

</xml_diff>

<commit_message>
Garantía DC-AG050: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -15950,7 +15950,11 @@
       <c r="J219" t="n">
         <v>68</v>
       </c>
-      <c r="K219" t="inlineStr"/>
+      <c r="K219" t="inlineStr">
+        <is>
+          <t>Destrucción</t>
+        </is>
+      </c>
       <c r="L219" t="inlineStr"/>
       <c r="M219" t="inlineStr"/>
       <c r="N219" t="inlineStr"/>
@@ -15972,10 +15976,14 @@
       <c r="T219" t="inlineStr"/>
       <c r="U219" t="inlineStr">
         <is>
-          <t>19/10/2026 11:03</t>
-        </is>
-      </c>
-      <c r="V219" t="inlineStr"/>
+          <t>19/10/2026 11:04</t>
+        </is>
+      </c>
+      <c r="V219" t="inlineStr">
+        <is>
+          <t>📨 Enviado a Cuentas por Pagar</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="1" t="n">
@@ -22891,7 +22899,11 @@
           <t>19/10/2026 11:03</t>
         </is>
       </c>
-      <c r="V327" t="inlineStr"/>
+      <c r="V327" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" s="1" t="n">

</xml_diff>

<commit_message>
Garantía DC-SEP043: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -22874,7 +22874,11 @@
       <c r="J327" t="n">
         <v>90</v>
       </c>
-      <c r="K327" t="inlineStr"/>
+      <c r="K327" t="inlineStr">
+        <is>
+          <t>Destrucción</t>
+        </is>
+      </c>
       <c r="L327" t="inlineStr"/>
       <c r="M327" t="inlineStr"/>
       <c r="N327" t="inlineStr"/>
@@ -22896,12 +22900,12 @@
       <c r="T327" t="inlineStr"/>
       <c r="U327" t="inlineStr">
         <is>
-          <t>19/10/2026 11:03</t>
+          <t>19/10/2026 11:04</t>
         </is>
       </c>
       <c r="V327" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-JL053: Folio marcado como RESUELTO (con NC, fecha cierre 08/10/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -12341,22 +12341,32 @@
       </c>
       <c r="L164" t="inlineStr"/>
       <c r="M164" t="inlineStr"/>
-      <c r="N164" t="inlineStr"/>
-      <c r="O164" t="inlineStr"/>
+      <c r="N164" t="inlineStr">
+        <is>
+          <t>369</t>
+        </is>
+      </c>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t>Descontado T-176451   nc-369  (Destruccion)</t>
+        </is>
+      </c>
       <c r="P164" s="1" t="n">
         <v>46252</v>
       </c>
       <c r="Q164" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R164" t="inlineStr"/>
       <c r="S164" t="inlineStr"/>
-      <c r="T164" t="inlineStr"/>
+      <c r="T164" s="1" t="n">
+        <v>46303</v>
+      </c>
       <c r="U164" t="inlineStr">
         <is>
-          <t>19/10/2026 11:03</t>
+          <t>19/10/2026 13:15</t>
         </is>
       </c>
       <c r="V164" t="inlineStr">

</xml_diff>

<commit_message>
Garantía DC-AG050: Folio marcado como RESUELTO (con NC, fecha cierre 08/10/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -15967,14 +15967,22 @@
       </c>
       <c r="L219" t="inlineStr"/>
       <c r="M219" t="inlineStr"/>
-      <c r="N219" t="inlineStr"/>
-      <c r="O219" t="inlineStr"/>
+      <c r="N219" t="inlineStr">
+        <is>
+          <t>369</t>
+        </is>
+      </c>
+      <c r="O219" t="inlineStr">
+        <is>
+          <t>Descontado T-176451   nc-369  (Destruccion)</t>
+        </is>
+      </c>
       <c r="P219" s="1" t="n">
         <v>46314</v>
       </c>
       <c r="Q219" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R219" s="1" t="n">
@@ -15983,10 +15991,12 @@
       <c r="S219" s="1" t="n">
         <v>46316</v>
       </c>
-      <c r="T219" t="inlineStr"/>
+      <c r="T219" s="1" t="n">
+        <v>46303</v>
+      </c>
       <c r="U219" t="inlineStr">
         <is>
-          <t>19/10/2026 11:04</t>
+          <t>19/10/2026 13:16</t>
         </is>
       </c>
       <c r="V219" t="inlineStr">

</xml_diff>

<commit_message>
Garantía DC-JN042: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -10975,7 +10975,11 @@
           <t>Recolección</t>
         </is>
       </c>
-      <c r="L145" t="inlineStr"/>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>8475</t>
+        </is>
+      </c>
       <c r="M145" t="inlineStr"/>
       <c r="N145" t="inlineStr"/>
       <c r="O145" t="inlineStr">
@@ -10994,7 +10998,11 @@
       <c r="R145" t="inlineStr"/>
       <c r="S145" t="inlineStr"/>
       <c r="T145" t="inlineStr"/>
-      <c r="U145" t="inlineStr"/>
+      <c r="U145" t="inlineStr">
+        <is>
+          <t>19/10/2026 14:13</t>
+        </is>
+      </c>
       <c r="V145" t="inlineStr">
         <is>
           <t>🗑️ En destrucción</t>

</xml_diff>

<commit_message>
Garantía DC-SEP004: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -823,7 +823,11 @@
       </c>
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -889,7 +893,11 @@
       </c>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -1169,7 +1177,11 @@
       </c>
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr"/>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -1313,7 +1325,11 @@
       </c>
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr"/>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -1533,7 +1549,11 @@
       </c>
       <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr"/>
-      <c r="V15" t="inlineStr"/>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -1599,7 +1619,11 @@
       </c>
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr"/>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -1825,7 +1849,11 @@
       </c>
       <c r="T19" t="inlineStr"/>
       <c r="U19" t="inlineStr"/>
-      <c r="V19" t="inlineStr"/>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
@@ -1891,7 +1919,11 @@
       </c>
       <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr"/>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -1957,7 +1989,11 @@
       </c>
       <c r="T21" t="inlineStr"/>
       <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr"/>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -2093,7 +2129,11 @@
       </c>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr"/>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
@@ -2609,7 +2649,11 @@
       </c>
       <c r="T30" t="inlineStr"/>
       <c r="U30" t="inlineStr"/>
-      <c r="V30" t="inlineStr"/>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
@@ -2971,7 +3015,11 @@
       </c>
       <c r="T35" t="inlineStr"/>
       <c r="U35" t="inlineStr"/>
-      <c r="V35" t="inlineStr"/>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
@@ -3181,7 +3229,11 @@
       </c>
       <c r="T38" t="inlineStr"/>
       <c r="U38" t="inlineStr"/>
-      <c r="V38" t="inlineStr"/>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
@@ -3561,7 +3613,11 @@
       </c>
       <c r="T43" t="inlineStr"/>
       <c r="U43" t="inlineStr"/>
-      <c r="V43" t="inlineStr"/>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
@@ -3627,7 +3683,11 @@
       </c>
       <c r="T44" t="inlineStr"/>
       <c r="U44" t="inlineStr"/>
-      <c r="V44" t="inlineStr"/>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
@@ -3693,7 +3753,11 @@
       </c>
       <c r="T45" t="inlineStr"/>
       <c r="U45" t="inlineStr"/>
-      <c r="V45" t="inlineStr"/>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
@@ -5117,7 +5181,11 @@
       </c>
       <c r="T64" t="inlineStr"/>
       <c r="U64" t="inlineStr"/>
-      <c r="V64" t="inlineStr"/>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
@@ -6373,7 +6441,11 @@
       </c>
       <c r="T81" t="inlineStr"/>
       <c r="U81" t="inlineStr"/>
-      <c r="V81" t="inlineStr"/>
+      <c r="V81" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="n">
@@ -6665,7 +6737,11 @@
       </c>
       <c r="T85" t="inlineStr"/>
       <c r="U85" t="inlineStr"/>
-      <c r="V85" t="inlineStr"/>
+      <c r="V85" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="n">
@@ -6803,7 +6879,11 @@
       </c>
       <c r="T87" t="inlineStr"/>
       <c r="U87" t="inlineStr"/>
-      <c r="V87" t="inlineStr"/>
+      <c r="V87" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="n">
@@ -6869,7 +6949,11 @@
       </c>
       <c r="T88" t="inlineStr"/>
       <c r="U88" t="inlineStr"/>
-      <c r="V88" t="inlineStr"/>
+      <c r="V88" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="n">
@@ -7893,7 +7977,11 @@
       </c>
       <c r="T102" t="inlineStr"/>
       <c r="U102" t="inlineStr"/>
-      <c r="V102" t="inlineStr"/>
+      <c r="V102" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
@@ -8335,7 +8423,11 @@
       </c>
       <c r="T108" t="inlineStr"/>
       <c r="U108" t="inlineStr"/>
-      <c r="V108" t="inlineStr"/>
+      <c r="V108" t="inlineStr">
+        <is>
+          <t>🚚 En recolección</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="1" t="n">
@@ -8401,7 +8493,11 @@
       </c>
       <c r="T109" t="inlineStr"/>
       <c r="U109" t="inlineStr"/>
-      <c r="V109" t="inlineStr"/>
+      <c r="V109" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="1" t="n">
@@ -9115,7 +9211,11 @@
       </c>
       <c r="T119" t="inlineStr"/>
       <c r="U119" t="inlineStr"/>
-      <c r="V119" t="inlineStr"/>
+      <c r="V119" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="n">
@@ -9181,7 +9281,11 @@
       </c>
       <c r="T120" t="inlineStr"/>
       <c r="U120" t="inlineStr"/>
-      <c r="V120" t="inlineStr"/>
+      <c r="V120" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="n">
@@ -10443,7 +10547,11 @@
       </c>
       <c r="T137" t="inlineStr"/>
       <c r="U137" t="inlineStr"/>
-      <c r="V137" t="inlineStr"/>
+      <c r="V137" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="n">
@@ -10509,7 +10617,11 @@
       </c>
       <c r="T138" t="inlineStr"/>
       <c r="U138" t="inlineStr"/>
-      <c r="V138" t="inlineStr"/>
+      <c r="V138" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="n">
@@ -10645,7 +10757,11 @@
       </c>
       <c r="T140" t="inlineStr"/>
       <c r="U140" t="inlineStr"/>
-      <c r="V140" t="inlineStr"/>
+      <c r="V140" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="n">
@@ -12143,7 +12259,11 @@
       </c>
       <c r="T161" t="inlineStr"/>
       <c r="U161" t="inlineStr"/>
-      <c r="V161" t="inlineStr"/>
+      <c r="V161" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="n">
@@ -12505,7 +12625,11 @@
       </c>
       <c r="T166" t="inlineStr"/>
       <c r="U166" t="inlineStr"/>
-      <c r="V166" t="inlineStr"/>
+      <c r="V166" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="n">
@@ -12853,7 +12977,11 @@
       </c>
       <c r="T171" t="inlineStr"/>
       <c r="U171" t="inlineStr"/>
-      <c r="V171" t="inlineStr"/>
+      <c r="V171" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="1" t="n">
@@ -13051,7 +13179,11 @@
       </c>
       <c r="T174" t="inlineStr"/>
       <c r="U174" t="inlineStr"/>
-      <c r="V174" t="inlineStr"/>
+      <c r="V174" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="1" t="n">
@@ -13175,7 +13307,11 @@
       </c>
       <c r="T176" t="inlineStr"/>
       <c r="U176" t="inlineStr"/>
-      <c r="V176" t="inlineStr"/>
+      <c r="V176" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="1" t="n">
@@ -13307,7 +13443,11 @@
       </c>
       <c r="T178" t="inlineStr"/>
       <c r="U178" t="inlineStr"/>
-      <c r="V178" t="inlineStr"/>
+      <c r="V178" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="1" t="n">
@@ -13369,7 +13509,11 @@
       </c>
       <c r="T179" t="inlineStr"/>
       <c r="U179" t="inlineStr"/>
-      <c r="V179" t="inlineStr"/>
+      <c r="V179" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="1" t="n">
@@ -13645,7 +13789,11 @@
       </c>
       <c r="T183" t="inlineStr"/>
       <c r="U183" t="inlineStr"/>
-      <c r="V183" t="inlineStr"/>
+      <c r="V183" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="1" t="n">
@@ -14091,7 +14239,11 @@
       </c>
       <c r="T190" t="inlineStr"/>
       <c r="U190" t="inlineStr"/>
-      <c r="V190" t="inlineStr"/>
+      <c r="V190" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="n">
@@ -14829,7 +14981,11 @@
       </c>
       <c r="T201" t="inlineStr"/>
       <c r="U201" t="inlineStr"/>
-      <c r="V201" t="inlineStr"/>
+      <c r="V201" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="1" t="n">
@@ -14891,7 +15047,11 @@
       </c>
       <c r="T202" t="inlineStr"/>
       <c r="U202" t="inlineStr"/>
-      <c r="V202" t="inlineStr"/>
+      <c r="V202" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="n">
@@ -14953,7 +15113,11 @@
       </c>
       <c r="T203" t="inlineStr"/>
       <c r="U203" t="inlineStr"/>
-      <c r="V203" t="inlineStr"/>
+      <c r="V203" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="1" t="n">
@@ -15015,7 +15179,11 @@
       </c>
       <c r="T204" t="inlineStr"/>
       <c r="U204" t="inlineStr"/>
-      <c r="V204" t="inlineStr"/>
+      <c r="V204" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="n">
@@ -15139,7 +15307,11 @@
       </c>
       <c r="T206" t="inlineStr"/>
       <c r="U206" t="inlineStr"/>
-      <c r="V206" t="inlineStr"/>
+      <c r="V206" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="1" t="n">
@@ -15395,7 +15567,11 @@
       </c>
       <c r="T210" t="inlineStr"/>
       <c r="U210" t="inlineStr"/>
-      <c r="V210" t="inlineStr"/>
+      <c r="V210" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="1" t="n">
@@ -15457,7 +15633,11 @@
       </c>
       <c r="T211" t="inlineStr"/>
       <c r="U211" t="inlineStr"/>
-      <c r="V211" t="inlineStr"/>
+      <c r="V211" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="1" t="n">
@@ -15519,7 +15699,11 @@
       </c>
       <c r="T212" t="inlineStr"/>
       <c r="U212" t="inlineStr"/>
-      <c r="V212" t="inlineStr"/>
+      <c r="V212" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="1" t="n">
@@ -15655,7 +15839,11 @@
       </c>
       <c r="T214" t="inlineStr"/>
       <c r="U214" t="inlineStr"/>
-      <c r="V214" t="inlineStr"/>
+      <c r="V214" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="1" t="n">
@@ -15717,7 +15905,11 @@
       </c>
       <c r="T215" t="inlineStr"/>
       <c r="U215" t="inlineStr"/>
-      <c r="V215" t="inlineStr"/>
+      <c r="V215" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="1" t="n">
@@ -16209,7 +16401,11 @@
       </c>
       <c r="T222" t="inlineStr"/>
       <c r="U222" t="inlineStr"/>
-      <c r="V222" t="inlineStr"/>
+      <c r="V222" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="1" t="n">
@@ -16333,7 +16529,11 @@
       </c>
       <c r="T224" t="inlineStr"/>
       <c r="U224" t="inlineStr"/>
-      <c r="V224" t="inlineStr"/>
+      <c r="V224" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="1" t="n">
@@ -16873,7 +17073,11 @@
       </c>
       <c r="T232" t="inlineStr"/>
       <c r="U232" t="inlineStr"/>
-      <c r="V232" t="inlineStr"/>
+      <c r="V232" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="1" t="n">
@@ -16935,7 +17139,11 @@
       </c>
       <c r="T233" t="inlineStr"/>
       <c r="U233" t="inlineStr"/>
-      <c r="V233" t="inlineStr"/>
+      <c r="V233" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="1" t="n">
@@ -17393,7 +17601,11 @@
       </c>
       <c r="T240" t="inlineStr"/>
       <c r="U240" t="inlineStr"/>
-      <c r="V240" t="inlineStr"/>
+      <c r="V240" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="1" t="n">
@@ -17919,7 +18131,11 @@
       </c>
       <c r="T248" t="inlineStr"/>
       <c r="U248" t="inlineStr"/>
-      <c r="V248" t="inlineStr"/>
+      <c r="V248" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="1" t="n">
@@ -17981,7 +18197,11 @@
       </c>
       <c r="T249" t="inlineStr"/>
       <c r="U249" t="inlineStr"/>
-      <c r="V249" t="inlineStr"/>
+      <c r="V249" t="inlineStr">
+        <is>
+          <t>📝 Reporte recibido</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="1" t="n">
@@ -20302,8 +20522,16 @@
       <c r="J285" t="n">
         <v>90</v>
       </c>
-      <c r="K285" t="inlineStr"/>
-      <c r="L285" t="inlineStr"/>
+      <c r="K285" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>8486</t>
+        </is>
+      </c>
       <c r="M285" t="inlineStr"/>
       <c r="N285" t="inlineStr"/>
       <c r="O285" t="inlineStr"/>
@@ -20318,10 +20546,14 @@
       <c r="R285" t="inlineStr"/>
       <c r="S285" t="inlineStr"/>
       <c r="T285" t="inlineStr"/>
-      <c r="U285" t="inlineStr"/>
+      <c r="U285" t="inlineStr">
+        <is>
+          <t>22/10/2026 15:28</t>
+        </is>
+      </c>
       <c r="V285" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-MZ011: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1300,8 +1300,16 @@
       <c r="J12" t="n">
         <v>16</v>
       </c>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>8478</t>
+        </is>
+      </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr">
@@ -1324,10 +1332,14 @@
         <v>46316</v>
       </c>
       <c r="T12" t="inlineStr"/>
-      <c r="U12" t="inlineStr"/>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>22/10/2026 15:48</t>
+        </is>
+      </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cuarentena: 1 folio(s) de CONEXIONES PLASTICAS DE AGUAS CALIENTES S.A DE C.V liberados (DC-SEP016)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -21358,11 +21358,11 @@
       <c r="N298" t="inlineStr"/>
       <c r="O298" t="inlineStr"/>
       <c r="P298" s="1" t="n">
-        <v>46312</v>
+        <v>46318</v>
       </c>
       <c r="Q298" t="inlineStr">
         <is>
-          <t>Cuarentena</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="R298" s="1" t="n">
@@ -21372,7 +21372,11 @@
         <v>46343</v>
       </c>
       <c r="T298" t="inlineStr"/>
-      <c r="U298" t="inlineStr"/>
+      <c r="U298" t="inlineStr">
+        <is>
+          <t>23/10/2026 17:43</t>
+        </is>
+      </c>
       <c r="V298" t="inlineStr"/>
     </row>
     <row r="299">

</xml_diff>

<commit_message>
Garantía DC-SEP016: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -21352,11 +21352,23 @@
       <c r="J298" t="n">
         <v>90</v>
       </c>
-      <c r="K298" t="inlineStr"/>
-      <c r="L298" t="inlineStr"/>
+      <c r="K298" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L298" t="inlineStr">
+        <is>
+          <t>8499</t>
+        </is>
+      </c>
       <c r="M298" t="inlineStr"/>
       <c r="N298" t="inlineStr"/>
-      <c r="O298" t="inlineStr"/>
+      <c r="O298" t="inlineStr">
+        <is>
+          <t>8499</t>
+        </is>
+      </c>
       <c r="P298" s="1" t="n">
         <v>46318</v>
       </c>
@@ -21374,10 +21386,14 @@
       <c r="T298" t="inlineStr"/>
       <c r="U298" t="inlineStr">
         <is>
-          <t>23/10/2026 17:43</t>
-        </is>
-      </c>
-      <c r="V298" t="inlineStr"/>
+          <t>23/10/2026 17:45</t>
+        </is>
+      </c>
+      <c r="V298" t="inlineStr">
+        <is>
+          <t>📨 Enviado a Cuentas por Pagar</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="n">

</xml_diff>

<commit_message>
Garantía DC-SEP038: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -22876,11 +22876,23 @@
       <c r="J322" t="n">
         <v>90</v>
       </c>
-      <c r="K322" t="inlineStr"/>
-      <c r="L322" t="inlineStr"/>
+      <c r="K322" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L322" t="inlineStr">
+        <is>
+          <t>8500</t>
+        </is>
+      </c>
       <c r="M322" t="inlineStr"/>
       <c r="N322" t="inlineStr"/>
-      <c r="O322" t="inlineStr"/>
+      <c r="O322" t="inlineStr">
+        <is>
+          <t>8500</t>
+        </is>
+      </c>
       <c r="P322" s="1" t="n">
         <v>46312</v>
       </c>
@@ -22892,10 +22904,14 @@
       <c r="R322" t="inlineStr"/>
       <c r="S322" t="inlineStr"/>
       <c r="T322" t="inlineStr"/>
-      <c r="U322" t="inlineStr"/>
+      <c r="U322" t="inlineStr">
+        <is>
+          <t>25/10/2026 23:16</t>
+        </is>
+      </c>
       <c r="V322" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-JL051: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -11912,11 +11912,23 @@
       <c r="J156" t="n">
         <v>38</v>
       </c>
-      <c r="K156" t="inlineStr"/>
-      <c r="L156" t="inlineStr"/>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>8475</t>
+        </is>
+      </c>
       <c r="M156" t="inlineStr"/>
       <c r="N156" t="inlineStr"/>
-      <c r="O156" t="inlineStr"/>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t>8475</t>
+        </is>
+      </c>
       <c r="P156" s="1" t="n">
         <v>46252</v>
       </c>
@@ -11928,10 +11940,14 @@
       <c r="R156" t="inlineStr"/>
       <c r="S156" t="inlineStr"/>
       <c r="T156" t="inlineStr"/>
-      <c r="U156" t="inlineStr"/>
+      <c r="U156" t="inlineStr">
+        <is>
+          <t>25/10/2026 23:23</t>
+        </is>
+      </c>
       <c r="V156" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-SEP062: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -24478,11 +24478,23 @@
       <c r="J347" t="n">
         <v>90</v>
       </c>
-      <c r="K347" t="inlineStr"/>
-      <c r="L347" t="inlineStr"/>
+      <c r="K347" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L347" t="inlineStr">
+        <is>
+          <t>8475</t>
+        </is>
+      </c>
       <c r="M347" t="inlineStr"/>
       <c r="N347" t="inlineStr"/>
-      <c r="O347" t="inlineStr"/>
+      <c r="O347" t="inlineStr">
+        <is>
+          <t>8575</t>
+        </is>
+      </c>
       <c r="P347" s="1" t="n">
         <v>46312</v>
       </c>
@@ -24494,10 +24506,14 @@
       <c r="R347" t="inlineStr"/>
       <c r="S347" t="inlineStr"/>
       <c r="T347" t="inlineStr"/>
-      <c r="U347" t="inlineStr"/>
+      <c r="U347" t="inlineStr">
+        <is>
+          <t>25/10/2026 23:35</t>
+        </is>
+      </c>
       <c r="V347" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-JL016: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -12134,11 +12134,23 @@
       <c r="J159" t="n">
         <v>38</v>
       </c>
-      <c r="K159" t="inlineStr"/>
-      <c r="L159" t="inlineStr"/>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>8498</t>
+        </is>
+      </c>
       <c r="M159" t="inlineStr"/>
       <c r="N159" t="inlineStr"/>
-      <c r="O159" t="inlineStr"/>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t>8498</t>
+        </is>
+      </c>
       <c r="P159" s="1" t="n">
         <v>46252</v>
       </c>
@@ -12150,10 +12162,14 @@
       <c r="R159" t="inlineStr"/>
       <c r="S159" t="inlineStr"/>
       <c r="T159" t="inlineStr"/>
-      <c r="U159" t="inlineStr"/>
+      <c r="U159" t="inlineStr">
+        <is>
+          <t>26/10/2026 01:18</t>
+        </is>
+      </c>
       <c r="V159" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-AG018: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -16084,11 +16084,23 @@
       <c r="J217" t="n">
         <v>68</v>
       </c>
-      <c r="K217" t="inlineStr"/>
-      <c r="L217" t="inlineStr"/>
+      <c r="K217" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L217" t="inlineStr">
+        <is>
+          <t>8498</t>
+        </is>
+      </c>
       <c r="M217" t="inlineStr"/>
       <c r="N217" t="inlineStr"/>
-      <c r="O217" t="inlineStr"/>
+      <c r="O217" t="inlineStr">
+        <is>
+          <t>8498</t>
+        </is>
+      </c>
       <c r="P217" s="1" t="n">
         <v>46282</v>
       </c>
@@ -16100,10 +16112,14 @@
       <c r="R217" t="inlineStr"/>
       <c r="S217" t="inlineStr"/>
       <c r="T217" t="inlineStr"/>
-      <c r="U217" t="inlineStr"/>
+      <c r="U217" t="inlineStr">
+        <is>
+          <t>26/10/2026 01:19</t>
+        </is>
+      </c>
       <c r="V217" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-JN010: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -19818,11 +19818,23 @@
       <c r="J273" t="n">
         <v>91</v>
       </c>
-      <c r="K273" t="inlineStr"/>
-      <c r="L273" t="inlineStr"/>
+      <c r="K273" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L273" t="inlineStr">
+        <is>
+          <t>8498</t>
+        </is>
+      </c>
       <c r="M273" t="inlineStr"/>
       <c r="N273" t="inlineStr"/>
-      <c r="O273" t="inlineStr"/>
+      <c r="O273" t="inlineStr">
+        <is>
+          <t>8498</t>
+        </is>
+      </c>
       <c r="P273" s="1" t="n">
         <v>46305</v>
       </c>
@@ -19834,10 +19846,14 @@
       <c r="R273" t="inlineStr"/>
       <c r="S273" t="inlineStr"/>
       <c r="T273" t="inlineStr"/>
-      <c r="U273" t="inlineStr"/>
+      <c r="U273" t="inlineStr">
+        <is>
+          <t>26/10/2026 01:19</t>
+        </is>
+      </c>
       <c r="V273" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-SEP020: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -21700,11 +21700,23 @@
       <c r="J302" t="n">
         <v>90</v>
       </c>
-      <c r="K302" t="inlineStr"/>
-      <c r="L302" t="inlineStr"/>
+      <c r="K302" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L302" t="inlineStr">
+        <is>
+          <t>8498</t>
+        </is>
+      </c>
       <c r="M302" t="inlineStr"/>
       <c r="N302" t="inlineStr"/>
-      <c r="O302" t="inlineStr"/>
+      <c r="O302" t="inlineStr">
+        <is>
+          <t>8498</t>
+        </is>
+      </c>
       <c r="P302" s="1" t="n">
         <v>46312</v>
       </c>
@@ -21716,10 +21728,14 @@
       <c r="R302" t="inlineStr"/>
       <c r="S302" t="inlineStr"/>
       <c r="T302" t="inlineStr"/>
-      <c r="U302" t="inlineStr"/>
+      <c r="U302" t="inlineStr">
+        <is>
+          <t>26/10/2026 01:20</t>
+        </is>
+      </c>
       <c r="V302" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-JL045: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -13206,11 +13206,23 @@
       <c r="J174" t="n">
         <v>38</v>
       </c>
-      <c r="K174" t="inlineStr"/>
-      <c r="L174" t="inlineStr"/>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>8495</t>
+        </is>
+      </c>
       <c r="M174" t="inlineStr"/>
       <c r="N174" t="inlineStr"/>
-      <c r="O174" t="inlineStr"/>
+      <c r="O174" t="inlineStr">
+        <is>
+          <t>8495</t>
+        </is>
+      </c>
       <c r="P174" s="1" t="n">
         <v>46316</v>
       </c>
@@ -13226,10 +13238,14 @@
         <v>46316</v>
       </c>
       <c r="T174" t="inlineStr"/>
-      <c r="U174" t="inlineStr"/>
+      <c r="U174" t="inlineStr">
+        <is>
+          <t>26/10/2026 01:25</t>
+        </is>
+      </c>
       <c r="V174" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-AG061: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -15750,11 +15750,23 @@
       <c r="J212" t="n">
         <v>68</v>
       </c>
-      <c r="K212" t="inlineStr"/>
-      <c r="L212" t="inlineStr"/>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L212" t="inlineStr">
+        <is>
+          <t>8496</t>
+        </is>
+      </c>
       <c r="M212" t="inlineStr"/>
       <c r="N212" t="inlineStr"/>
-      <c r="O212" t="inlineStr"/>
+      <c r="O212" t="inlineStr">
+        <is>
+          <t>8496</t>
+        </is>
+      </c>
       <c r="P212" s="1" t="n">
         <v>46316</v>
       </c>
@@ -15770,10 +15782,14 @@
         <v>46316</v>
       </c>
       <c r="T212" t="inlineStr"/>
-      <c r="U212" t="inlineStr"/>
+      <c r="U212" t="inlineStr">
+        <is>
+          <t>26/10/2026 01:29</t>
+        </is>
+      </c>
       <c r="V212" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cuarentena: 1 folio(s) de PERFIHERRAJES IMMSA SA DE CV liberados (DC-SEP048)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -23642,11 +23642,11 @@
       <c r="N332" t="inlineStr"/>
       <c r="O332" t="inlineStr"/>
       <c r="P332" s="1" t="n">
-        <v>46312</v>
+        <v>46321</v>
       </c>
       <c r="Q332" t="inlineStr">
         <is>
-          <t>Cuarentena</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="R332" s="1" t="n">
@@ -23656,7 +23656,11 @@
         <v>46343</v>
       </c>
       <c r="T332" t="inlineStr"/>
-      <c r="U332" t="inlineStr"/>
+      <c r="U332" t="inlineStr">
+        <is>
+          <t>26/10/2026 01:30</t>
+        </is>
+      </c>
       <c r="V332" t="inlineStr"/>
     </row>
     <row r="333">

</xml_diff>

<commit_message>
Garantía DC-SEP048: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -23636,11 +23636,23 @@
       <c r="J332" t="n">
         <v>90</v>
       </c>
-      <c r="K332" t="inlineStr"/>
-      <c r="L332" t="inlineStr"/>
+      <c r="K332" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L332" t="inlineStr">
+        <is>
+          <t>8496</t>
+        </is>
+      </c>
       <c r="M332" t="inlineStr"/>
       <c r="N332" t="inlineStr"/>
-      <c r="O332" t="inlineStr"/>
+      <c r="O332" t="inlineStr">
+        <is>
+          <t>8496</t>
+        </is>
+      </c>
       <c r="P332" s="1" t="n">
         <v>46321</v>
       </c>
@@ -23658,10 +23670,14 @@
       <c r="T332" t="inlineStr"/>
       <c r="U332" t="inlineStr">
         <is>
-          <t>26/10/2026 01:30</t>
-        </is>
-      </c>
-      <c r="V332" t="inlineStr"/>
+          <t>26/10/2026 01:31</t>
+        </is>
+      </c>
+      <c r="V332" t="inlineStr">
+        <is>
+          <t>📨 Enviado a Cuentas por Pagar</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" s="1" t="n">

</xml_diff>

<commit_message>
Cuarentena: 1 folio(s) de INDUSTRIAL MEXICANA DE HERRAMIENTAS S.A. DE C.V. liberados (DC-SEP027)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -22250,11 +22250,11 @@
       <c r="N310" t="inlineStr"/>
       <c r="O310" t="inlineStr"/>
       <c r="P310" s="1" t="n">
-        <v>46312</v>
+        <v>46321</v>
       </c>
       <c r="Q310" t="inlineStr">
         <is>
-          <t>Cuarentena</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="R310" s="1" t="n">
@@ -22264,7 +22264,11 @@
         <v>46343</v>
       </c>
       <c r="T310" t="inlineStr"/>
-      <c r="U310" t="inlineStr"/>
+      <c r="U310" t="inlineStr">
+        <is>
+          <t>26/10/2026 01:39</t>
+        </is>
+      </c>
       <c r="V310" t="inlineStr"/>
     </row>
     <row r="311">

</xml_diff>

<commit_message>
Garantía DC-SEP027: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -22252,11 +22252,23 @@
       <c r="J310" t="n">
         <v>90</v>
       </c>
-      <c r="K310" t="inlineStr"/>
-      <c r="L310" t="inlineStr"/>
+      <c r="K310" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L310" t="inlineStr">
+        <is>
+          <t>8494</t>
+        </is>
+      </c>
       <c r="M310" t="inlineStr"/>
       <c r="N310" t="inlineStr"/>
-      <c r="O310" t="inlineStr"/>
+      <c r="O310" t="inlineStr">
+        <is>
+          <t>8494</t>
+        </is>
+      </c>
       <c r="P310" s="1" t="n">
         <v>46321</v>
       </c>
@@ -22274,12 +22286,12 @@
       <c r="T310" t="inlineStr"/>
       <c r="U310" t="inlineStr">
         <is>
-          <t>26/10/2026 01:39</t>
+          <t>26/10/2026 01:41</t>
         </is>
       </c>
       <c r="V310" t="inlineStr">
         <is>
-          <t>📝 Reporte recibido</t>
+          <t>📨 Enviado a Cuentas por Pagar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garantía DC-MY042: Folio marcado como RESUELTO (con NC, fecha cierre 22/09/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -19102,23 +19102,45 @@
       <c r="J261" t="n">
         <v>91</v>
       </c>
-      <c r="K261" t="inlineStr"/>
-      <c r="L261" t="inlineStr"/>
+      <c r="K261" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L261" t="inlineStr">
+        <is>
+          <t>8367</t>
+        </is>
+      </c>
       <c r="M261" t="inlineStr"/>
-      <c r="N261" t="inlineStr"/>
-      <c r="O261" t="inlineStr"/>
+      <c r="N261" t="inlineStr">
+        <is>
+          <t>48936</t>
+        </is>
+      </c>
+      <c r="O261" t="inlineStr">
+        <is>
+          <t>ajuste 48936 cambio fisico</t>
+        </is>
+      </c>
       <c r="P261" s="1" t="n">
         <v>46305</v>
       </c>
       <c r="Q261" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R261" t="inlineStr"/>
       <c r="S261" t="inlineStr"/>
-      <c r="T261" t="inlineStr"/>
-      <c r="U261" t="inlineStr"/>
+      <c r="T261" s="1" t="n">
+        <v>46287</v>
+      </c>
+      <c r="U261" t="inlineStr">
+        <is>
+          <t>26/10/2026 11:45</t>
+        </is>
+      </c>
       <c r="V261" t="inlineStr">
         <is>
           <t>📝 Reporte recibido</t>

</xml_diff>

<commit_message>
Garantía DC-JN031: Folio marcado como RESUELTO (con NC, fecha cierre 22/09/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -20292,23 +20292,45 @@
       <c r="J279" t="n">
         <v>91</v>
       </c>
-      <c r="K279" t="inlineStr"/>
-      <c r="L279" t="inlineStr"/>
+      <c r="K279" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L279" t="inlineStr">
+        <is>
+          <t>8367</t>
+        </is>
+      </c>
       <c r="M279" t="inlineStr"/>
-      <c r="N279" t="inlineStr"/>
-      <c r="O279" t="inlineStr"/>
+      <c r="N279" t="inlineStr">
+        <is>
+          <t>48936</t>
+        </is>
+      </c>
+      <c r="O279" t="inlineStr">
+        <is>
+          <t>ajuste 48936 cambio fisico</t>
+        </is>
+      </c>
       <c r="P279" s="1" t="n">
         <v>46305</v>
       </c>
       <c r="Q279" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R279" t="inlineStr"/>
       <c r="S279" t="inlineStr"/>
-      <c r="T279" t="inlineStr"/>
-      <c r="U279" t="inlineStr"/>
+      <c r="T279" s="1" t="n">
+        <v>46287</v>
+      </c>
+      <c r="U279" t="inlineStr">
+        <is>
+          <t>26/10/2026 11:46</t>
+        </is>
+      </c>
       <c r="V279" t="inlineStr">
         <is>
           <t>📝 Reporte recibido</t>

</xml_diff>

<commit_message>
Cuarentena: 1 folio(s) de METALURGICA BALFE SA DE CV liberados (DC-SEP045)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -23540,11 +23540,11 @@
       <c r="N329" t="inlineStr"/>
       <c r="O329" t="inlineStr"/>
       <c r="P329" s="1" t="n">
-        <v>46312</v>
+        <v>46321</v>
       </c>
       <c r="Q329" t="inlineStr">
         <is>
-          <t>Cuarentena</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="R329" s="1" t="n">
@@ -23554,7 +23554,11 @@
         <v>46343</v>
       </c>
       <c r="T329" t="inlineStr"/>
-      <c r="U329" t="inlineStr"/>
+      <c r="U329" t="inlineStr">
+        <is>
+          <t>26/10/2026 11:48</t>
+        </is>
+      </c>
       <c r="V329" t="inlineStr"/>
     </row>
     <row r="330">

</xml_diff>

<commit_message>
Garantía DC-SEP045: Cambios guardados
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -23534,11 +23534,23 @@
       <c r="J329" t="n">
         <v>90</v>
       </c>
-      <c r="K329" t="inlineStr"/>
-      <c r="L329" t="inlineStr"/>
+      <c r="K329" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
+      <c r="L329" t="inlineStr">
+        <is>
+          <t>8497</t>
+        </is>
+      </c>
       <c r="M329" t="inlineStr"/>
       <c r="N329" t="inlineStr"/>
-      <c r="O329" t="inlineStr"/>
+      <c r="O329" t="inlineStr">
+        <is>
+          <t>8497</t>
+        </is>
+      </c>
       <c r="P329" s="1" t="n">
         <v>46321</v>
       </c>
@@ -23556,10 +23568,14 @@
       <c r="T329" t="inlineStr"/>
       <c r="U329" t="inlineStr">
         <is>
-          <t>26/10/2026 11:48</t>
-        </is>
-      </c>
-      <c r="V329" t="inlineStr"/>
+          <t>26/10/2026 11:49</t>
+        </is>
+      </c>
+      <c r="V329" t="inlineStr">
+        <is>
+          <t>📨 Enviado a Cuentas por Pagar</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" s="1" t="n">

</xml_diff>

<commit_message>
Garantía DC-JL052: Folio marcado como RESUELTO (con NC, fecha cierre 25/09/2026)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -12733,10 +12733,14 @@
         </is>
       </c>
       <c r="M167" t="inlineStr"/>
-      <c r="N167" t="inlineStr"/>
+      <c r="N167" t="inlineStr">
+        <is>
+          <t>175926</t>
+        </is>
+      </c>
       <c r="O167" t="inlineStr">
         <is>
-          <t>8439 Devolucion</t>
+          <t>8439 Devolucion    descontado en la transferencia 175926</t>
         </is>
       </c>
       <c r="P167" s="1" t="n">
@@ -12744,15 +12748,17 @@
       </c>
       <c r="Q167" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Resuelto</t>
         </is>
       </c>
       <c r="R167" t="inlineStr"/>
       <c r="S167" t="inlineStr"/>
-      <c r="T167" t="inlineStr"/>
+      <c r="T167" s="1" t="n">
+        <v>46290</v>
+      </c>
       <c r="U167" t="inlineStr">
         <is>
-          <t>05/10/2026 02:32</t>
+          <t>26/10/2026 15:13</t>
         </is>
       </c>
       <c r="V167" t="inlineStr">

</xml_diff>